<commit_message>
docs(srs): align SRS and tracker with architecture decisions
Bump the SRS to v0.2: sync the data model with the ERD (sessions,
driver_profiles, zone code keys, pool capacity snapshot), record
decisions D-13 to D-23 with ADR links and resolve open issues OI-01
to OI-03. Mirror the new decisions and task/requirement statuses in
the traceability workbook.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements_RTM'!$A$1:$O$138</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test_Cases'!$A$1:$K$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Assumptions_Decisions'!$A$1:$I$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Assumptions_Decisions'!$A$1:$I$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Implementation_Tasks'!$A$1:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'State_Transitions'!$A$1:$G$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Glossary'!$A$1:$B$16</definedName>
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="B2:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -688,7 +688,6 @@
     <col width="4" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -703,7 +702,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -724,7 +722,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>0.1 (Draft for review)</t>
+          <t>0.2 (Draft for review) — see SRS revision history</t>
         </is>
       </c>
     </row>
@@ -764,7 +762,18 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Last updated</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-24 — architecture phase: ARCHITECTURE.md, ERD.md, ADR-0001…0012</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
         <is>
@@ -844,7 +853,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1010,7 +1018,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
@@ -1227,7 +1234,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
@@ -8101,7 +8107,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="N86" s="16" t="inlineStr"/>
+      <c r="N86" s="16" t="inlineStr">
+        <is>
+          <t>Mechanism designed: ARCHITECTURE.md §7, ADR-0006</t>
+        </is>
+      </c>
       <c r="O86" s="16" t="inlineStr"/>
       <c r="P86" s="4">
         <f>","&amp;SUBSTITUTE(F86," ","")&amp;","</f>
@@ -10926,10 +10936,14 @@
       </c>
       <c r="M126" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N126" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N126" s="16" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md §3–4, §12; docs/ERD.md §1</t>
+        </is>
+      </c>
       <c r="O126" s="16" t="inlineStr"/>
       <c r="P126" s="4">
         <f>","&amp;SUBSTITUTE(F126," ","")&amp;","</f>
@@ -10995,10 +11009,14 @@
       </c>
       <c r="M127" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N127" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N127" s="16" t="inlineStr">
+        <is>
+          <t>docs/adr/0001–0012 (README summary pending, T-24)</t>
+        </is>
+      </c>
       <c r="O127" s="16" t="inlineStr"/>
       <c r="P127" s="4">
         <f>","&amp;SUBSTITUTE(F127," ","")&amp;","</f>
@@ -11765,7 +11783,11 @@
           <t>In Progress</t>
         </is>
       </c>
-      <c r="N138" s="16" t="inlineStr"/>
+      <c r="N138" s="16" t="inlineStr">
+        <is>
+          <t>SRS v0.2 revision 2026-09-24</t>
+        </is>
+      </c>
       <c r="O138" s="16" t="inlineStr"/>
       <c r="P138" s="4">
         <f>","&amp;SUBSTITUTE(F138," ","")&amp;","</f>
@@ -14182,7 +14204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15510,7 +15532,7 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>PostgreSQL is recommended as the DBMS. The final choice and justification belong to the architecture phase.</t>
+          <t>The DBMS is PostgreSQL 16 (ADR-0002).</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -15520,12 +15542,12 @@
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>MySQL, SQLite</t>
+          <t>MySQL, SQLite, MongoDB</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
-          <t>DC-03, NFR-CON-04</t>
+          <t>DC-03, NFR-CON-04, ADR-0002</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr">
@@ -15543,38 +15565,42 @@
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>D-14</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>PRD inconsistency</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>The PRD mandates a master branch, but the repository was initialised with main.</t>
+          <t>The system is a modular monolith: Next.js web + one Express API + PostgreSQL (ADR-0001).</t>
         </is>
       </c>
       <c r="D33" s="17" t="inlineStr">
         <is>
-          <t>Create master and use it as the integration branch (DR-01).</t>
-        </is>
-      </c>
-      <c r="E33" s="17" t="inlineStr"/>
+          <t>Every invariant fits in one ACID transaction, with no distributed consistency (PRD §9).</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Next.js-only; microservices</t>
+        </is>
+      </c>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t>DR-01</t>
+          <t>DC-05, DR-14</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Proposed</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I33" s="16" t="inlineStr"/>
@@ -15582,200 +15608,642 @@
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
+          <t>D-15</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>The API is built with Express 5 + TypeScript (ADR-0003).</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>No hidden control flow, a large ecosystem, and explicit layering that is simple to trace and maintain.</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>NestJS; Fastify</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>DC-02, DC-07</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>Chosen by product owner in architecture session</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>D-16</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Data access uses Prisma, with CHECK constraints, partial unique indexes and triggers in hand-written SQL migrations (ADR-0004).</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Type-safe DX for most queries. Raw SQL is visible exactly where the integrity guarantees are implemented.</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Drizzle; Knex; TypeORM</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>NFR-CON-04, NFR-POR-03, NFR-SEC-08</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <t>Chosen by product owner in architecture session</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>D-17</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Auth uses opaque DB-backed sessions (SHA-256 hash stored) in an httpOnly cookie, behind a same-origin Next.js /api proxy (ADR-0005).</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Real logout; a DB leak exposes no usable tokens; first-party cookies across different hosts.</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>JWT in cookie; Auth.js/Lucia</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>FR-AUTH-02, FR-AUTH-03, NFR-SEC-06</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H36" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Chosen by product owner in architecture session</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="63" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>D-18</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>Concurrency uses row locks in the fixed order driver → pool → ride → wallet, compare-and-set transitions and DB constraints. Expiry is checked in the accept CAS, plus a 60 s in-process sweeper (ADR-0006).</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>Deterministic outcome for the last-seat race, with no extra infrastructure.</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Optimistic versioning; SERIALIZABLE; Redis lock</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>NFR-CON-01, NFR-CON-02, NFR-CON-03, NFR-REL-04</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr"/>
+    </row>
+    <row r="38" ht="33" customHeight="1">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>D-19</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>The repo is an npm-workspaces monorepo: apps/web, apps/api, packages/shared (Zod, enums, transition tables) (ADR-0008).</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>One source for schemas, enums and transition tables across web and API.</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Turborepo/Nx; two repos</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>NFR-MNT-01, NFR-MNT-03</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39" ht="48" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>D-20</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>Deployment is Docker Compose now, then Vercel + Railway + Supabase on free tiers, with a verify-no-payment guardrail (ADR-0009).</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>The primary run path (docker compose up) never depends on third parties, and the same images run in the cloud.</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>Render-only; Vercel + Render + Neon</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>NFR-POR-01, NFR-POR-04, DC-04, DR-11</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I39" s="16" t="inlineStr">
+        <is>
+          <t>Chosen by product owner in architecture session</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="33" customHeight="1">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>D-21</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Tests use Vitest + Supertest against a real PostgreSQL test DB (ADR-0011).</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Locks and constraints can only be proven against the real engine.</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Jest; mocks/SQLite; Testcontainers</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>DR-10, NFR-MNT-04</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="H40" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41" ht="33" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>D-22</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>The frontend uses the Next.js App Router + TanStack Query (polling) + react-hook-form + Tailwind CSS (ADR-0012).</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>Built-in loading/error states and polling; a small, maintainable UI stack.</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>Vite + React Router; SWR; component libraries</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>DC-01, FR-PAX-07, NFR-USA-01</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I41" s="16" t="inlineStr"/>
+    </row>
+    <row r="42" ht="48" customHeight="1">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>D-23</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>Schema choices: pool_members link table, pools.capacity snapshot, driver_profiles table, zone code natural key, UUID ids, polymorphic append-only status_history (ERD §8).</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Row-local CHECK for capacity, re-matching history, driver-only ownership that is structural.</t>
+        </is>
+      </c>
+      <c r="E42" s="13" t="inlineStr">
+        <is>
+          <t>ride_requests.pool_id; capacity via trigger; driver columns on users</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>FR-POOL-02, FR-POOL-10, FR-HIST-02</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I42" s="16" t="inlineStr"/>
+    </row>
+    <row r="43" ht="33" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>PRD inconsistency</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>The PRD mandates a master branch, but the repository was initialised with main.</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>Create master and use it as the integration branch (DR-01).</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="n"/>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>DR-01</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="I43" s="16" t="n"/>
+    </row>
+    <row r="44" ht="33" customHeight="1">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
           <t>P-02</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>PRD inconsistency</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
         <is>
           <t>PRD §18 refers to "the concurrency problem in Section 14". It is actually in §12.</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D44" s="13" t="inlineStr">
         <is>
           <t>Treated as §12.</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr"/>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E44" s="13" t="n"/>
+      <c r="F44" s="13" t="inlineStr">
         <is>
           <t>NFR-CON-01</t>
         </is>
       </c>
-      <c r="G34" s="15" t="inlineStr">
+      <c r="G44" s="15" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
       </c>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="H44" s="14" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="I34" s="16" t="inlineStr"/>
-    </row>
-    <row r="35" ht="33" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="I44" s="16" t="n"/>
+    </row>
+    <row r="45" ht="33" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>P-03</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>PRD inconsistency</t>
         </is>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C45" s="17" t="inlineStr">
         <is>
           <t>The PRD lifecycle mixes passenger-level and trip-level states.</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D45" s="17" t="inlineStr">
         <is>
           <t>Split into two state machines (D-12).</t>
         </is>
       </c>
-      <c r="E35" s="17" t="inlineStr"/>
-      <c r="F35" s="17" t="inlineStr">
+      <c r="E45" s="17" t="n"/>
+      <c r="F45" s="17" t="inlineStr">
         <is>
           <t>§5</t>
         </is>
       </c>
-      <c r="G35" s="15" t="inlineStr">
+      <c r="G45" s="15" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
       </c>
-      <c r="H35" s="9" t="inlineStr">
+      <c r="H45" s="9" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="I35" s="16" t="inlineStr"/>
-    </row>
-    <row r="36" ht="33" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="I45" s="16" t="n"/>
+    </row>
+    <row r="46" ht="33" customHeight="1">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>OI-01</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>Open issue</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>Choose the backend framework, ORM, auth mechanism, test framework, styling and hosting, each justified per DC-07.</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>Resolve in: Architecture phase</t>
-        </is>
-      </c>
-      <c r="E36" s="13" t="inlineStr"/>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>Resolved 2026-09-24: D-14…D-22, ADR-0001…0012</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="n"/>
+      <c r="F46" s="13" t="inlineStr">
         <is>
           <t>DC-07, DR-07</t>
         </is>
       </c>
-      <c r="G36" s="15" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="H36" s="14" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="I36" s="16" t="inlineStr"/>
-    </row>
-    <row r="37" ht="48" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="H46" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I46" s="16" t="n"/>
+    </row>
+    <row r="47" ht="48" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>OI-02</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>Open issue</t>
         </is>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="C47" s="17" t="inlineStr">
         <is>
           <t>Choose the concrete concurrency mechanism (pessimistic SELECT … FOR UPDATE versus a conditional update guarded by CHECK) and document it.</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
-        <is>
-          <t>Resolve in: Architecture phase</t>
-        </is>
-      </c>
-      <c r="E37" s="17" t="inlineStr"/>
-      <c r="F37" s="17" t="inlineStr">
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>Resolved 2026-09-24: row locks + CAS + constraints in layers (D-18, ADR-0006)</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="n"/>
+      <c r="F47" s="17" t="inlineStr">
         <is>
           <t>NFR-CON-03</t>
         </is>
       </c>
-      <c r="G37" s="15" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="H37" s="9" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="I37" s="16" t="inlineStr"/>
-    </row>
-    <row r="38" ht="48" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I47" s="16" t="n"/>
+    </row>
+    <row r="48" ht="48" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>OI-03</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B48" s="14" t="inlineStr">
         <is>
           <t>Open issue</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>Decide whether the request-expiry sweeper runs as an in-process interval or lazily on read (NFR-REL-04 requires lazy correctness either way).</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>Resolve in: Architecture phase</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr"/>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>Resolved 2026-09-24: expiry checked in accept CAS, plus 60 s in-process sweeper (D-18)</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="n"/>
+      <c r="F48" s="13" t="inlineStr">
         <is>
           <t>NFR-REL-04</t>
         </is>
       </c>
-      <c r="G38" s="15" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="H38" s="14" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="I38" s="16" t="inlineStr"/>
+      <c r="G48" s="15" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="H48" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I48" s="16" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I38"/>
+  <autoFilter ref="A1:I48"/>
   <conditionalFormatting sqref="G2:G237">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$G2="Proposed"</formula>
@@ -15905,7 +16373,11 @@
         </is>
       </c>
       <c r="H2" s="16" t="inlineStr"/>
-      <c r="I2" s="16" t="inlineStr"/>
+      <c r="I2" s="16" t="inlineStr">
+        <is>
+          <t>SRS v0.2 synced with ERD on 2026-09-24</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="33" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -15938,11 +16410,19 @@
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="inlineStr"/>
-      <c r="I3" s="16" t="inlineStr"/>
+          <t>In Review</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md, docs/ERD.md, docs/adr/0001–0012</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>Drafted 2026-09-24; awaiting review</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="33" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -17611,7 +18091,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
@@ -17799,7 +18278,6 @@
       <c r="G28" s="19" t="inlineStr"/>
       <c r="H28" s="19" t="inlineStr"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
@@ -18216,7 +18694,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -18651,7 +19128,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -18713,7 +19189,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -18766,8 +19241,6 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -19326,7 +19799,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: sync architecture, ERD and tracker with the project setup
Point ARCHITECTURE at SRS v0.3 and record what the setup introduced:
config/rules.ts and logger.ts in the repository layout, Node-based
container health checks on node:24-bookworm-slim images, and the
DB_PORT variable. Correct the ERD revision note to 15 tables.

Tracker: mark T-03 to T-05 done with commit evidence, update the
requirements they implement, record TC-34 as partially written, and
move T-14 to feature/tesla-pooling (accept needs driver availability).
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="B2:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -688,7 +688,6 @@
     <col width="4" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -703,7 +702,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -772,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — same-gender ride option (BR-18) added; architecture phase docs (ARCHITECTURE.md, ERD.md, ADR-0001…0012)</t>
+          <t>2026-09-24 — Phase 0 (feature/project-setup): monorepo, conventions, API foundation, Docker</t>
         </is>
       </c>
     </row>
@@ -855,7 +853,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1021,7 +1018,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
@@ -1238,7 +1234,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
@@ -3302,7 +3297,7 @@
       </c>
       <c r="L20" s="13" t="inlineStr">
         <is>
-          <t>feature/driver-flow, feature/driver-ui</t>
+          <t>feature/tesla-pooling, feature/driver-ui</t>
         </is>
       </c>
       <c r="M20" s="15" t="inlineStr">
@@ -3375,7 +3370,7 @@
       </c>
       <c r="L21" s="17" t="inlineStr">
         <is>
-          <t>feature/driver-flow, feature/driver-ui</t>
+          <t>feature/tesla-pooling, feature/driver-ui</t>
         </is>
       </c>
       <c r="M21" s="15" t="inlineStr">
@@ -3448,7 +3443,7 @@
       </c>
       <c r="L22" s="13" t="inlineStr">
         <is>
-          <t>feature/driver-flow</t>
+          <t>feature/tesla-pooling</t>
         </is>
       </c>
       <c r="M22" s="15" t="inlineStr">
@@ -3521,7 +3516,7 @@
       </c>
       <c r="L23" s="17" t="inlineStr">
         <is>
-          <t>feature/driver-flow, feature/driver-ui</t>
+          <t>feature/tesla-pooling, feature/driver-ui</t>
         </is>
       </c>
       <c r="M23" s="15" t="inlineStr">
@@ -7845,10 +7840,14 @@
       </c>
       <c r="M82" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N82" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N82" s="16" t="inlineStr">
+        <is>
+          <t>ZodError → VALIDATION_ERROR mapping in error handler; schemas per endpoint later</t>
+        </is>
+      </c>
       <c r="O82" s="16" t="inlineStr"/>
       <c r="P82" s="4">
         <f>","&amp;SUBSTITUTE(F82," ","")&amp;","</f>
@@ -7918,10 +7917,14 @@
       </c>
       <c r="M83" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N83" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N83" s="16" t="inlineStr">
+        <is>
+          <t>.gitignore excludes .env; .env.example placeholders only — commits f221565, 7d59b8d</t>
+        </is>
+      </c>
       <c r="O83" s="16" t="inlineStr"/>
       <c r="P83" s="4">
         <f>","&amp;SUBSTITUTE(F83," ","")&amp;","</f>
@@ -7991,10 +7994,14 @@
       </c>
       <c r="M84" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N84" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N84" s="16" t="inlineStr">
+        <is>
+          <t>helmet headers + CORS to WEB_ORIGIN done; session cookie flags in feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O84" s="16" t="inlineStr"/>
       <c r="P84" s="4">
         <f>","&amp;SUBSTITUTE(F84," ","")&amp;","</f>
@@ -8214,10 +8221,14 @@
       </c>
       <c r="M87" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N87" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N87" s="16" t="inlineStr">
+        <is>
+          <t>Generic INTERNAL_ERROR message; details only in logs — commit 51da796</t>
+        </is>
+      </c>
       <c r="O87" s="16" t="inlineStr"/>
       <c r="P87" s="4">
         <f>","&amp;SUBSTITUTE(F87," ","")&amp;","</f>
@@ -8729,10 +8740,14 @@
       </c>
       <c r="M94" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N94" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N94" s="16" t="inlineStr">
+        <is>
+          <t>middleware/error-handler.ts; test/app.test.ts — commit 51da796</t>
+        </is>
+      </c>
       <c r="O94" s="16" t="inlineStr"/>
       <c r="P94" s="4">
         <f>","&amp;SUBSTITUTE(F94," ","")&amp;","</f>
@@ -8802,10 +8817,14 @@
       </c>
       <c r="M95" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N95" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N95" s="16" t="inlineStr">
+        <is>
+          <t>/health + compose health checks — commits 51da796, 7d59b8d</t>
+        </is>
+      </c>
       <c r="O95" s="16" t="inlineStr"/>
       <c r="P95" s="4">
         <f>","&amp;SUBSTITUTE(F95," ","")&amp;","</f>
@@ -9678,10 +9697,14 @@
       </c>
       <c r="M107" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N107" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N107" s="16" t="inlineStr">
+        <is>
+          <t>docker compose up works (3 healthy); migrations/seed arrive in feature/db-schema</t>
+        </is>
+      </c>
       <c r="O107" s="16" t="inlineStr"/>
       <c r="P107" s="4">
         <f>","&amp;SUBSTITUTE(F107," ","")&amp;","</f>
@@ -9747,10 +9770,14 @@
       </c>
       <c r="M108" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N108" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N108" s="16" t="inlineStr">
+        <is>
+          <t>config/env.ts, config/rules.ts, .env.example — commits 9ddba2e, 51da796, 7d59b8d</t>
+        </is>
+      </c>
       <c r="O108" s="16" t="inlineStr"/>
       <c r="P108" s="4">
         <f>","&amp;SUBSTITUTE(F108," ","")&amp;","</f>
@@ -9962,10 +9989,14 @@
       </c>
       <c r="M111" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N111" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N111" s="16" t="inlineStr">
+        <is>
+          <t>logger.ts, middleware/http-logger.ts — commits 51da796, 28caad4</t>
+        </is>
+      </c>
       <c r="O111" s="16" t="inlineStr"/>
       <c r="P111" s="4">
         <f>","&amp;SUBSTITUTE(F111," ","")&amp;","</f>
@@ -10100,10 +10131,14 @@
       </c>
       <c r="M113" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N113" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N113" s="16" t="inlineStr">
+        <is>
+          <t>pino redaction; headers not logged — commit 28caad4</t>
+        </is>
+      </c>
       <c r="O113" s="16" t="inlineStr"/>
       <c r="P113" s="4">
         <f>","&amp;SUBSTITUTE(F113," ","")&amp;","</f>
@@ -10169,10 +10204,14 @@
       </c>
       <c r="M114" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N114" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N114" s="16" t="inlineStr">
+        <is>
+          <t>Module template documented (CODING_CONVENTIONS §4); health module follows it</t>
+        </is>
+      </c>
       <c r="O114" s="16" t="inlineStr"/>
       <c r="P114" s="4">
         <f>","&amp;SUBSTITUTE(F114," ","")&amp;","</f>
@@ -10311,10 +10350,14 @@
       </c>
       <c r="M116" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N116" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N116" s="16" t="inlineStr">
+        <is>
+          <t>TypeScript strict, ESLint (simplicity rules), Prettier — commit f221565</t>
+        </is>
+      </c>
       <c r="O116" s="16" t="inlineStr"/>
       <c r="P116" s="4">
         <f>","&amp;SUBSTITUTE(F116," ","")&amp;","</f>
@@ -10380,10 +10423,14 @@
       </c>
       <c r="M117" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N117" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N117" s="16" t="inlineStr">
+        <is>
+          <t>npm test at root and in Docker (docker compose run --rm api npm test)</t>
+        </is>
+      </c>
       <c r="O117" s="16" t="inlineStr"/>
       <c r="P117" s="4">
         <f>","&amp;SUBSTITUTE(F117," ","")&amp;","</f>
@@ -10449,10 +10496,14 @@
       </c>
       <c r="M118" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N118" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N118" s="16" t="inlineStr">
+        <is>
+          <t>apps/web: Next.js App Router</t>
+        </is>
+      </c>
       <c r="O118" s="16" t="inlineStr"/>
       <c r="P118" s="4">
         <f>","&amp;SUBSTITUTE(F118," ","")&amp;","</f>
@@ -10518,10 +10569,14 @@
       </c>
       <c r="M119" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N119" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N119" s="16" t="inlineStr">
+        <is>
+          <t>apps/api: Node.js + Express 5</t>
+        </is>
+      </c>
       <c r="O119" s="16" t="inlineStr"/>
       <c r="P119" s="4">
         <f>","&amp;SUBSTITUTE(F119," ","")&amp;","</f>
@@ -10587,10 +10642,14 @@
       </c>
       <c r="M120" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N120" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N120" s="16" t="inlineStr">
+        <is>
+          <t>PostgreSQL 16 container</t>
+        </is>
+      </c>
       <c r="O120" s="16" t="inlineStr"/>
       <c r="P120" s="4">
         <f>","&amp;SUBSTITUTE(F120," ","")&amp;","</f>
@@ -10725,10 +10784,14 @@
       </c>
       <c r="M122" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N122" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N122" s="16" t="inlineStr">
+        <is>
+          <t>Three containers only: db, api, web</t>
+        </is>
+      </c>
       <c r="O122" s="16" t="inlineStr"/>
       <c r="P122" s="4">
         <f>","&amp;SUBSTITUTE(F122," ","")&amp;","</f>
@@ -10794,10 +10857,14 @@
       </c>
       <c r="M123" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N123" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N123" s="16" t="inlineStr">
+        <is>
+          <t>No third-party runtime services</t>
+        </is>
+      </c>
       <c r="O123" s="16" t="inlineStr"/>
       <c r="P123" s="4">
         <f>","&amp;SUBSTITUTE(F123," ","")&amp;","</f>
@@ -11508,10 +11575,14 @@
       </c>
       <c r="M133" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N133" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N133" s="16" t="inlineStr">
+        <is>
+          <t>docker-compose.yml and .env.example added; migrations/seed in feature/db-schema</t>
+        </is>
+      </c>
       <c r="O133" s="16" t="inlineStr"/>
       <c r="P133" s="4">
         <f>","&amp;SUBSTITUTE(F133," ","")&amp;","</f>
@@ -13933,11 +14004,19 @@
       </c>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J35" s="16" t="inlineStr"/>
-      <c r="K35" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J35" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/app.test.ts (404, malformed JSON, requestId); 409/500 cases added with later modules</t>
+        </is>
+      </c>
+      <c r="K35" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="33" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
@@ -17245,11 +17324,19 @@
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H4" s="16" t="inlineStr"/>
-      <c r="I4" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>f221565 chore(repo), 9ddba2e docs(conventions) on feature/project-setup</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Also added docs/CODING_CONVENTIONS.md and config/rules.ts</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -17282,11 +17369,19 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="inlineStr"/>
-      <c r="I5" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>51da796 feat(api), 28caad4 refactor(api) on feature/project-setup</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>Tests: apps/api/test/app.test.ts</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -17319,11 +17414,19 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="inlineStr"/>
-      <c r="I6" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>7d59b8d build(docker) on feature/project-setup</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Verified: 3 containers healthy, web page shows 'API ok', tests pass in container</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -17629,7 +17732,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>feature/driver-flow</t>
+          <t>feature/tesla-pooling</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
@@ -17656,7 +17759,11 @@
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr"/>
-      <c r="I15" s="16" t="inlineStr"/>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Moved from feature/driver-flow: accept needs driver availability first (plan Phase 5)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="63" customHeight="1">
       <c r="A16" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync ERD and tracker with the database schema
ERD v0.3 records what the implemented schema settled: the nullable
wallet_transactions.reason column that marks the SEED opening
balance, status_history.id as an auto-increment bigint, and the names
of the two migration files.

Tracker: mark T-06 and T-07 done with commit evidence, update the
requirements the schema, integrity migration and seed implement, and
record TC-07 and TC-37 as passing locally and in Docker.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 0 (feature/project-setup): monorepo, conventions, API foundation, Docker</t>
+          <t>2026-09-24 — Phase 1 (feature/db-schema): schema, integrity migration, db helpers, seed, constraint tests</t>
         </is>
       </c>
     </row>
@@ -2361,10 +2361,14 @@
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N7" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N7" s="16" t="inlineStr">
+        <is>
+          <t>Jashim/Bullet and Kamal/Toofan seeded — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O7" s="16" t="inlineStr"/>
       <c r="P7" s="4">
         <f>","&amp;SUBSTITUTE(F7," ","")&amp;","</f>
@@ -4835,10 +4839,14 @@
       </c>
       <c r="M41" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N41" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N41" s="16" t="inlineStr">
+        <is>
+          <t>pool_members_one_active_membership index tested; accept flow in feature/tesla-pooling — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O41" s="16" t="inlineStr"/>
       <c r="P41" s="4">
         <f>","&amp;SUBSTITUTE(F41," ","")&amp;","</f>
@@ -4908,10 +4916,14 @@
       </c>
       <c r="M42" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N42" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N42" s="16" t="inlineStr">
+        <is>
+          <t>pool_members table; roster endpoint in feature/driver-flow — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O42" s="16" t="inlineStr"/>
       <c r="P42" s="4">
         <f>","&amp;SUBSTITUTE(F42," ","")&amp;","</f>
@@ -5500,10 +5512,14 @@
       </c>
       <c r="M50" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N50" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N50" s="16" t="inlineStr">
+        <is>
+          <t>All money columns BIGINT paisa; formatting in UI later — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O50" s="16" t="inlineStr"/>
       <c r="P50" s="4">
         <f>","&amp;SUBSTITUTE(F50," ","")&amp;","</f>
@@ -5938,10 +5954,14 @@
       </c>
       <c r="M56" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N56" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N56" s="16" t="inlineStr">
+        <is>
+          <t>wallets_balance_check + append-only ledger tested; settlement in feature/teslapay-wallet — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O56" s="16" t="inlineStr"/>
       <c r="P56" s="4">
         <f>","&amp;SUBSTITUTE(F56," ","")&amp;","</f>
@@ -6084,10 +6104,14 @@
       </c>
       <c r="M58" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N58" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N58" s="16" t="inlineStr">
+        <is>
+          <t>Append-only trigger tested; audit writer in feature/ride-request — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O58" s="16" t="inlineStr"/>
       <c r="P58" s="4">
         <f>","&amp;SUBSTITUTE(F58," ","")&amp;","</f>
@@ -6741,10 +6765,14 @@
       </c>
       <c r="M67" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N67" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N67" s="16" t="inlineStr">
+        <is>
+          <t>prisma/seed-data/zones.ts; symmetry test — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O67" s="16" t="inlineStr"/>
       <c r="P67" s="4">
         <f>","&amp;SUBSTITUTE(F67," ","")&amp;","</f>
@@ -7252,10 +7280,14 @@
       </c>
       <c r="M74" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N74" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N74" s="16" t="inlineStr">
+        <is>
+          <t>BIGINT *_paisa columns; db/money.ts exact conversion — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O74" s="16" t="inlineStr"/>
       <c r="P74" s="4">
         <f>","&amp;SUBSTITUTE(F74," ","")&amp;","</f>
@@ -8144,12 +8176,12 @@
       </c>
       <c r="M86" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="N86" s="16" t="inlineStr">
         <is>
-          <t>Mechanism designed: ARCHITECTURE.md §7, ADR-0006</t>
+          <t>Prisma query API + tagged $queryRaw only — feature/db-schema</t>
         </is>
       </c>
       <c r="O86" s="16" t="inlineStr"/>
@@ -8521,10 +8553,14 @@
       </c>
       <c r="M91" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N91" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N91" s="16" t="inlineStr">
+        <is>
+          <t>Partial unique indexes; test/db/constraints.test.ts — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O91" s="16" t="inlineStr"/>
       <c r="P91" s="4">
         <f>","&amp;SUBSTITUTE(F91," ","")&amp;","</f>
@@ -9113,10 +9149,14 @@
       </c>
       <c r="M99" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N99" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N99" s="16" t="inlineStr">
+        <is>
+          <t>Indexes in init + integrity migrations (ERD §5) — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O99" s="16" t="inlineStr"/>
       <c r="P99" s="4">
         <f>","&amp;SUBSTITUTE(F99," ","")&amp;","</f>
@@ -9697,12 +9737,12 @@
       </c>
       <c r="M107" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>docker compose up works (3 healthy); migrations/seed arrive in feature/db-schema</t>
+          <t>Fresh volume: migrate deploy → seed → API healthy; web healthy — feature/db-schema</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr"/>
@@ -9847,10 +9887,14 @@
       </c>
       <c r="M109" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N109" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N109" s="16" t="inlineStr">
+        <is>
+          <t>Versioned migrations; idempotent seed (test/db/seed.test.ts) — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O109" s="16" t="inlineStr"/>
       <c r="P109" s="4">
         <f>","&amp;SUBSTITUTE(F109," ","")&amp;","</f>
@@ -11575,12 +11619,12 @@
       </c>
       <c r="M133" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N133" s="16" t="inlineStr">
         <is>
-          <t>docker-compose.yml and .env.example added; migrations/seed in feature/db-schema</t>
+          <t>docker-compose.yml, .env.example, migrations, persona seed — feature/project-setup, feature/db-schema</t>
         </is>
       </c>
       <c r="O133" s="16" t="inlineStr"/>
@@ -12005,10 +12049,14 @@
       </c>
       <c r="M139" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N139" s="16" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N139" s="16" t="inlineStr">
+        <is>
+          <t>Personas in seed and test helpers — feature/db-schema</t>
+        </is>
+      </c>
       <c r="O139" s="16" t="n"/>
       <c r="P139" s="4">
         <f>","&amp;SUBSTITUTE(F139," ","")&amp;","</f>
@@ -12681,11 +12729,19 @@
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J8" s="16" t="inlineStr"/>
-      <c r="K8" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/db/constraints.test.ts</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -14159,11 +14215,19 @@
       </c>
       <c r="I38" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J38" s="16" t="inlineStr"/>
-      <c r="K38" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J38" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/db/seed.test.ts (automated; no user1/driver1 in seed data)</t>
+        </is>
+      </c>
+      <c r="K38" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
@@ -17459,11 +17523,19 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H7" s="16" t="inlineStr"/>
-      <c r="I7" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>e7db6c7 feat(db) schema, 77d5ab5 feat(db) integrity migration, 5c0b0e9 feat(db) helpers — feature/db-schema</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Prisma migrate diff shows no drift against the hand-written objects</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -17496,11 +17568,19 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr"/>
-      <c r="I8" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>b9272b5 feat(seed) — feature/db-schema</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Seed runs on container start; idempotent (TC-37)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, env example and tracker with the auth module
Architecture v0.4 records that the login rate limit is keyed on the
client IP behind exactly one trusted proxy hop and that sign-out
returns 204. Document SESSION_TTL_HOURS and COOKIE_SECURE in
.env.example.

Tracker: mark T-08 and T-09 done, record the auth, session and
security requirements they implement, and mark TC-31, TC-32, TC-38 and
TC-44 as passing (TC-04 and TC-50 partly written).
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 1 (feature/db-schema): schema, integrity migration, db helpers, seed, constraint tests</t>
+          <t>2026-09-24 — Phase 2 (feature/passenger-auth): shared schemas, sign-up/sign-in, sessions, guards, rate limit</t>
         </is>
       </c>
     </row>
@@ -1996,10 +1996,14 @@
       </c>
       <c r="M2" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N2" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N2" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/auth/signup; test/auth/sign-up.test.ts — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O2" s="16" t="inlineStr"/>
       <c r="P2" s="4">
         <f>","&amp;SUBSTITUTE(F2," ","")&amp;","</f>
@@ -2069,10 +2073,14 @@
       </c>
       <c r="M3" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N3" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N3" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/auth/login (e-mail or phone); test/auth/sessions.test.ts — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O3" s="16" t="inlineStr"/>
       <c r="P3" s="4">
         <f>","&amp;SUBSTITUTE(F3," ","")&amp;","</f>
@@ -2142,10 +2150,14 @@
       </c>
       <c r="M4" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N4" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/auth/logout revokes the session — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O4" s="16" t="inlineStr"/>
       <c r="P4" s="4">
         <f>","&amp;SUBSTITUTE(F4," ","")&amp;","</f>
@@ -2215,10 +2227,14 @@
       </c>
       <c r="M5" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N5" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N5" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/auth/me (vehicle for drivers) — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O5" s="16" t="inlineStr"/>
       <c r="P5" s="4">
         <f>","&amp;SUBSTITUTE(F5," ","")&amp;","</f>
@@ -2288,10 +2304,14 @@
       </c>
       <c r="M6" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N6" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N6" s="16" t="inlineStr">
+        <is>
+          <t>API role guards done (test/auth/access.test.ts); web routing in feature/passenger-ui — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O6" s="16" t="inlineStr"/>
       <c r="P6" s="4">
         <f>","&amp;SUBSTITUTE(F6," ","")&amp;","</f>
@@ -7653,10 +7673,14 @@
       </c>
       <c r="M79" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N79" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N79" s="16" t="inlineStr">
+        <is>
+          <t>bcrypt (cost 12; 4 in tests); TC-44 — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O79" s="16" t="inlineStr"/>
       <c r="P79" s="4">
         <f>","&amp;SUBSTITUTE(F79," ","")&amp;","</f>
@@ -7726,10 +7750,14 @@
       </c>
       <c r="M80" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N80" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N80" s="16" t="inlineStr">
+        <is>
+          <t>requireAuth in place; applied to each new endpoint as modules arrive — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O80" s="16" t="inlineStr"/>
       <c r="P80" s="4">
         <f>","&amp;SUBSTITUTE(F80," ","")&amp;","</f>
@@ -7799,10 +7827,14 @@
       </c>
       <c r="M81" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N81" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N81" s="16" t="inlineStr">
+        <is>
+          <t>Role guards done; object-level ownership checks with rides/pools — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O81" s="16" t="inlineStr"/>
       <c r="P81" s="4">
         <f>","&amp;SUBSTITUTE(F81," ","")&amp;","</f>
@@ -7877,7 +7909,7 @@
       </c>
       <c r="N82" s="16" t="inlineStr">
         <is>
-          <t>ZodError → VALIDATION_ERROR mapping in error handler; schemas per endpoint later</t>
+          <t>validateBody with strict shared schemas for auth; other endpoints later — feature/passenger-auth</t>
         </is>
       </c>
       <c r="O82" s="16" t="inlineStr"/>
@@ -8026,12 +8058,12 @@
       </c>
       <c r="M84" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N84" s="16" t="inlineStr">
         <is>
-          <t>helmet headers + CORS to WEB_ORIGIN done; session cookie flags in feature/passenger-auth</t>
+          <t>httpOnly SameSite=Lax cookie (Secure via COOKIE_SECURE), helmet, CORS — feature/passenger-auth</t>
         </is>
       </c>
       <c r="O84" s="16" t="inlineStr"/>
@@ -8103,10 +8135,14 @@
       </c>
       <c r="M85" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N85" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N85" s="16" t="inlineStr">
+        <is>
+          <t>express-rate-limit 10/min per IP; TC-38 — feature/passenger-auth</t>
+        </is>
+      </c>
       <c r="O85" s="16" t="inlineStr"/>
       <c r="P85" s="4">
         <f>","&amp;SUBSTITUTE(F85," ","")&amp;","</f>
@@ -12582,11 +12618,19 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J5" s="16" t="inlineStr"/>
-      <c r="K5" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Role part in test/auth/access.test.ts; ride/pool ownership with those modules</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 partial</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -13913,11 +13957,19 @@
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J32" s="16" t="inlineStr"/>
-      <c r="K32" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J32" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/auth/sign-up.test.ts</t>
+        </is>
+      </c>
+      <c r="K32" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
@@ -13962,11 +14014,19 @@
       </c>
       <c r="I33" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J33" s="16" t="inlineStr"/>
-      <c r="K33" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J33" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/auth/sessions.test.ts</t>
+        </is>
+      </c>
+      <c r="K33" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
@@ -14272,11 +14332,19 @@
       </c>
       <c r="I39" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J39" s="16" t="inlineStr"/>
-      <c r="K39" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J39" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/auth/rate-limit.test.ts</t>
+        </is>
+      </c>
+      <c r="K39" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="33" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
@@ -14566,11 +14634,19 @@
       </c>
       <c r="I45" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J45" s="16" t="inlineStr"/>
-      <c r="K45" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J45" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/auth/sessions.test.ts (automated: bcrypt hashes, SHA-256 token hash)</t>
+        </is>
+      </c>
+      <c r="K45" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="33" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
@@ -14860,11 +14936,19 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J51" s="16" t="inlineStr"/>
-      <c r="K51" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J51" s="16" t="inlineStr">
+        <is>
+          <t>Part 1 (gender optional at sign-up) in test/auth/sign-up.test.ts; option validation with rides</t>
+        </is>
+      </c>
+      <c r="K51" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 partial</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="14" t="inlineStr">
@@ -17613,11 +17697,19 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="inlineStr"/>
-      <c r="I9" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>6ee7875 feat(shared), 0fccd56 feat(auth), 347e153 feat(auth) — feature/passenger-auth</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Sign-up, sign-in, sessions, sign-out, /me</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="33" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -17650,11 +17742,19 @@
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="inlineStr"/>
-      <c r="I10" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>347e153 feat(auth) guards, cea26a4 feat(auth) rate limit, 07b28b6 test(auth) — feature/passenger-auth</t>
+        </is>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>requireAuth/requireRole; 10 attempts/min per IP behind one trusted proxy hop</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, conventions and tracker with the fare module
ARCHITECTURE v0.5: the domain layer may use shared types; zone data is cached in memory; the fare breakdown shape, CURRENT_FARE_RATES and roundHalfUpDiv are documented; the test folder layout matches the code. The conventions guide explains how to change the fare rates. Tracker: T-10 and T-11 done; FR-PAX-01, FR-FARE-01, BR-09, BR-10, BR-11 and BR-13 implemented; TC-03, TC-10, TC-12 and TC-35 passing.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 2 (feature/passenger-auth): shared schemas, sign-up/sign-in, sessions, guards, rate limit</t>
+          <t>2026-09-24 — Phase 3 (feature/zones-fares): fare calculator in paisa, zones and fare-estimate endpoints</t>
         </is>
       </c>
     </row>
@@ -2519,10 +2519,14 @@
       </c>
       <c r="M9" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N9" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N9" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/zones; test/zones/zones.test.ts — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O9" s="16" t="inlineStr"/>
       <c r="P9" s="4">
         <f>","&amp;SUBSTITUTE(F9," ","")&amp;","</f>
@@ -2592,10 +2596,14 @@
       </c>
       <c r="M10" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N10" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N10" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/fares/estimate returns solo and pooled (TC-35); form in feature/passenger-ui — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O10" s="16" t="inlineStr"/>
       <c r="P10" s="4">
         <f>","&amp;SUBSTITUTE(F10," ","")&amp;","</f>
@@ -5167,10 +5175,14 @@
       </c>
       <c r="M45" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N45" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N45" s="16" t="inlineStr">
+        <is>
+          <t>domain/fare.ts computeFare; test/domain/fare.test.ts (TC-03, TC-12) — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O45" s="16" t="inlineStr"/>
       <c r="P45" s="4">
         <f>","&amp;SUBSTITUTE(F45," ","")&amp;","</f>
@@ -5240,10 +5252,14 @@
       </c>
       <c r="M46" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N46" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N46" s="16" t="inlineStr">
+        <is>
+          <t>Estimate returns both figures; stored on the request in feature/ride-request — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O46" s="16" t="inlineStr"/>
       <c r="P46" s="4">
         <f>","&amp;SUBSTITUTE(F46," ","")&amp;","</f>
@@ -5386,10 +5402,14 @@
       </c>
       <c r="M48" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N48" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N48" s="16" t="inlineStr">
+        <is>
+          <t>API returns base, distance charge, discount, seats, total (TC-35); views in the UI branches — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O48" s="16" t="inlineStr"/>
       <c r="P48" s="4">
         <f>","&amp;SUBSTITUTE(F48," ","")&amp;","</f>
@@ -5537,7 +5557,7 @@
       </c>
       <c r="N50" s="16" t="inlineStr">
         <is>
-          <t>All money columns BIGINT paisa; formatting in UI later — feature/db-schema</t>
+          <t>BIGINT paisa columns (feature/db-schema); integer-only fare arithmetic in domain/money.ts (feature/zones-fares); display formatting in the UI</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr"/>
@@ -6935,10 +6955,14 @@
       </c>
       <c r="M69" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N69" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N69" s="16" t="inlineStr">
+        <is>
+          <t>zones.service distanceBetween from the seeded table (TC-12) — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O69" s="16" t="inlineStr"/>
       <c r="P69" s="4">
         <f>","&amp;SUBSTITUTE(F69," ","")&amp;","</f>
@@ -7008,10 +7032,14 @@
       </c>
       <c r="M70" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N70" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N70" s="16" t="inlineStr">
+        <is>
+          <t>domain/fare.ts; TC-03, TC-10, TC-12 — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O70" s="16" t="inlineStr"/>
       <c r="P70" s="4">
         <f>","&amp;SUBSTITUTE(F70," ","")&amp;","</f>
@@ -7081,10 +7109,14 @@
       </c>
       <c r="M71" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N71" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N71" s="16" t="inlineStr">
+        <is>
+          <t>FARE_* env rates via config/rules.ts CURRENT_FARE_RATES; base never discounted (test) — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O71" s="16" t="inlineStr"/>
       <c r="P71" s="4">
         <f>","&amp;SUBSTITUTE(F71," ","")&amp;","</f>
@@ -7154,10 +7186,14 @@
       </c>
       <c r="M72" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N72" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N72" s="16" t="inlineStr">
+        <is>
+          <t>computeFare takes the pooled flag (TC-10: 2 seats of 1 passenger not pooled); locking at start in feature/driver-flow — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O72" s="16" t="inlineStr"/>
       <c r="P72" s="4">
         <f>","&amp;SUBSTITUTE(F72," ","")&amp;","</f>
@@ -7227,10 +7263,14 @@
       </c>
       <c r="M73" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N73" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N73" s="16" t="inlineStr">
+        <is>
+          <t>roundHalfUpDiv on the integer remainder; test/domain/money.test.ts — feature/zones-fares</t>
+        </is>
+      </c>
       <c r="O73" s="16" t="inlineStr"/>
       <c r="P73" s="4">
         <f>","&amp;SUBSTITUTE(F73," ","")&amp;","</f>
@@ -7909,7 +7949,7 @@
       </c>
       <c r="N82" s="16" t="inlineStr">
         <is>
-          <t>validateBody with strict shared schemas for auth; other endpoints later — feature/passenger-auth</t>
+          <t>validateBody with strict shared schemas for auth and fare estimates; unexpected fields named in the 400 — feature/zones-fares</t>
         </is>
       </c>
       <c r="O82" s="16" t="inlineStr"/>
@@ -12569,11 +12609,19 @@
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J4" s="16" t="inlineStr"/>
-      <c r="K4" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/domain/fare.test.ts</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -12928,11 +12976,19 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="inlineStr"/>
-      <c r="K11" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/domain/fare.test.ts (fare level); trip-start check with feature/driver-flow</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -13026,11 +13082,19 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="inlineStr"/>
-      <c r="K13" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/domain/fare.test.ts, test/zones/zones.test.ts, test/fares/estimate.test.ts</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
@@ -14177,11 +14241,19 @@
       </c>
       <c r="I36" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J36" s="16" t="inlineStr"/>
-      <c r="K36" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J36" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/zones/zones.test.ts, apps/api/test/fares/estimate.test.ts</t>
+        </is>
+      </c>
+      <c r="K36" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="33" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
@@ -17787,11 +17859,19 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H11" s="16" t="inlineStr"/>
-      <c r="I11" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>b4e67b9 feat(fare), 1be55c0 test(fare), d9ff25f test(fare) — feature/zones-fares</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>computeFare() and roundHalfUpDiv() on whole paisa; rates from CURRENT_FARE_RATES</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -17824,11 +17904,19 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H12" s="16" t="inlineStr"/>
-      <c r="I12" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>2a5c39d feat(fare), 86a24c5 fix(api), 63be8bb test(fare) — feature/zones-fares</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/zones, POST /api/fares/estimate; zone reference data cached in memory</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, conventions and tracker with the rides module
ARCHITECTURE v0.6: transition tables live in the shared package; the rides, audit and wallet function names match the code; cancellation.ts is listed; §6.1 and §7.3 show that a passenger's overdue rides are expired in their own transaction before each command; refused commands are logged as command.rejected. The conventions guide explains how to allow a new status change. Tracker: T-12 done, T-13 in progress; FR-PAX-03…05, BR-05, BR-06, FR-HIST-02, FR-HIST-03, NFR-OBS-02, NFR-MNT-02 and NFR-CON-06 implemented; TC-08, TC-18, TC-33 and TC-39 passing.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 3 (feature/zones-fares): fare calculator in paisa, zones and fare-estimate endpoints</t>
+          <t>2026-09-24 — Phase 4 (feature/ride-request): state machines, audit trail, ride requests, expiry, unmatched cancellation</t>
         </is>
       </c>
     </row>
@@ -2673,10 +2673,14 @@
       </c>
       <c r="M11" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N11" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/rides; test/rides/request.test.ts (TC-33) — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O11" s="16" t="inlineStr"/>
       <c r="P11" s="4">
         <f>","&amp;SUBSTITUTE(F11," ","")&amp;","</f>
@@ -2746,10 +2750,14 @@
       </c>
       <c r="M12" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N12" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N12" s="16" t="inlineStr">
+        <is>
+          <t>409 ACTIVE_REQUEST_EXISTS with the existing ride id; double submit covered (TC-18) — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O12" s="16" t="inlineStr"/>
       <c r="P12" s="4">
         <f>","&amp;SUBSTITUTE(F12," ","")&amp;","</f>
@@ -2819,10 +2827,14 @@
       </c>
       <c r="M13" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N13" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N13" s="16" t="inlineStr">
+        <is>
+          <t>422 INSUFFICIENT_BALANCE against the solo estimate; Rafiq test — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O13" s="16" t="inlineStr"/>
       <c r="P13" s="4">
         <f>","&amp;SUBSTITUTE(F13," ","")&amp;","</f>
@@ -2892,10 +2904,14 @@
       </c>
       <c r="M14" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N14" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N14" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/rides?scope=active and /:id with driver, Tesla, co-rider count, badge — feature/ride-request; screen in feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O14" s="16" t="inlineStr"/>
       <c r="P14" s="4">
         <f>","&amp;SUBSTITUTE(F14," ","")&amp;","</f>
@@ -3038,10 +3054,14 @@
       </c>
       <c r="M16" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N16" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N16" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/rides/:id/cancel: REQUESTED free, STARTED/terminal 409 — feature/ride-request; MATCHED and DRIVER_ARRIVED (fee) later</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr"/>
       <c r="P16" s="4">
         <f>","&amp;SUBSTITUTE(F16," ","")&amp;","</f>
@@ -3111,10 +3131,14 @@
       </c>
       <c r="M17" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N17" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/rides?scope=history, newest first, cursor paging (TC-39) — feature/ride-request; screen in feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O17" s="16" t="inlineStr"/>
       <c r="P17" s="4">
         <f>","&amp;SUBSTITUTE(F17," ","")&amp;","</f>
@@ -3184,10 +3208,14 @@
       </c>
       <c r="M18" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N18" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N18" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/rides/:id timeline from status_history — feature/ride-request; screen in feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr"/>
       <c r="P18" s="4">
         <f>","&amp;SUBSTITUTE(F18," ","")&amp;","</f>
@@ -3257,10 +3285,14 @@
       </c>
       <c r="M19" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N19" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>Option validation (TC-50 parts 2-3) — feature/ride-request; matching in feature/tesla-pooling, badge in the UI</t>
+        </is>
+      </c>
       <c r="O19" s="16" t="inlineStr">
         <is>
           <t>Added in SRS v0.3</t>
@@ -5252,12 +5284,12 @@
       </c>
       <c r="M46" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N46" s="16" t="inlineStr">
         <is>
-          <t>Estimate returns both figures; stored on the request in feature/ride-request — feature/zones-fares</t>
+          <t>Estimate endpoint (feature/zones-fares); estimated_fare_paisa stored on each request and both figures in the ride view — feature/ride-request</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr"/>
@@ -6071,10 +6103,14 @@
       </c>
       <c r="M57" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N57" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N57" s="16" t="inlineStr">
+        <is>
+          <t>recordTransition in the same transaction: ride create, cancel, expiry — feature/ride-request; pool and driver transitions follow</t>
+        </is>
+      </c>
       <c r="O57" s="16" t="inlineStr"/>
       <c r="P57" s="4">
         <f>","&amp;SUBSTITUTE(F57," ","")&amp;","</f>
@@ -6144,12 +6180,12 @@
       </c>
       <c r="M58" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N58" s="16" t="inlineStr">
         <is>
-          <t>Append-only trigger tested; audit writer in feature/ride-request — feature/db-schema</t>
+          <t>Append-only trigger (feature/db-schema); audit module has no update/delete path — feature/ride-request</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr"/>
@@ -6221,10 +6257,14 @@
       </c>
       <c r="M59" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N59" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N59" s="16" t="inlineStr">
+        <is>
+          <t>error-handler logs 409/422 at WARN as command.rejected with code and request id — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O59" s="16" t="inlineStr"/>
       <c r="P59" s="4">
         <f>","&amp;SUBSTITUTE(F59," ","")&amp;","</f>
@@ -6294,10 +6334,14 @@
       </c>
       <c r="M60" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N60" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N60" s="16" t="inlineStr">
+        <is>
+          <t>Ride, timeline and fare rows readable per ride — feature/ride-request; full E1 reconstruction after feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O60" s="16" t="inlineStr"/>
       <c r="P60" s="4">
         <f>","&amp;SUBSTITUTE(F60," ","")&amp;","</f>
@@ -6659,10 +6703,14 @@
       </c>
       <c r="M65" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N65" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N65" s="16" t="inlineStr">
+        <is>
+          <t>Service check plus partial unique index; TC-18 — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O65" s="16" t="inlineStr"/>
       <c r="P65" s="4">
         <f>","&amp;SUBSTITUTE(F65," ","")&amp;","</f>
@@ -6732,10 +6780,14 @@
       </c>
       <c r="M66" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N66" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N66" s="16" t="inlineStr">
+        <is>
+          <t>domain/state-machine.ts over shared transition tables; TC-08 exhaustive — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O66" s="16" t="inlineStr"/>
       <c r="P66" s="4">
         <f>","&amp;SUBSTITUTE(F66," ","")&amp;","</f>
@@ -6882,10 +6934,14 @@
       </c>
       <c r="M68" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N68" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N68" s="16" t="inlineStr">
+        <is>
+          <t>domain/cancellation.ts policy (FREE/FEE/FORBIDDEN); fee charging in feature/driver-flow — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O68" s="16" t="inlineStr"/>
       <c r="P68" s="4">
         <f>","&amp;SUBSTITUTE(F68," ","")&amp;","</f>
@@ -7872,7 +7928,7 @@
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Role guards done; object-level ownership checks with rides/pools — feature/passenger-auth</t>
+          <t>Role guards (feature/passenger-auth); rides scoped to their owner, 404 for others (TC-04 part) — feature/ride-request</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr"/>
@@ -7949,7 +8005,7 @@
       </c>
       <c r="N82" s="16" t="inlineStr">
         <is>
-          <t>validateBody with strict shared schemas for auth and fare estimates; unexpected fields named in the 400 — feature/zones-fares</t>
+          <t>validateBody with strict shared schemas for auth, estimates and rides; list query parsed with Zod — feature/ride-request</t>
         </is>
       </c>
       <c r="O82" s="16" t="inlineStr"/>
@@ -8479,10 +8535,14 @@
       </c>
       <c r="M89" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N89" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N89" s="16" t="inlineStr">
+        <is>
+          <t>CAS on status for cancel and expiry, audit in the same transaction — feature/ride-request; accept/pool moves in feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O89" s="16" t="inlineStr"/>
       <c r="P89" s="4">
         <f>","&amp;SUBSTITUTE(F89," ","")&amp;","</f>
@@ -8779,10 +8839,14 @@
       </c>
       <c r="M93" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N93" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N93" s="16" t="inlineStr">
+        <is>
+          <t>Relies on NFR-CON-04: a retry gets 409 ACTIVE_REQUEST_EXISTS with the original ride id — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O93" s="16" t="inlineStr"/>
       <c r="P93" s="4">
         <f>","&amp;SUBSTITUTE(F93," ","")&amp;","</f>
@@ -9079,10 +9143,14 @@
       </c>
       <c r="M97" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N97" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N97" s="16" t="inlineStr">
+        <is>
+          <t>Expiry on read and before every passenger command, plus the 60 s sweep — feature/ride-request; accept check in feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O97" s="16" t="inlineStr"/>
       <c r="P97" s="4">
         <f>","&amp;SUBSTITUTE(F97," ","")&amp;","</f>
@@ -10182,10 +10250,14 @@
       </c>
       <c r="M112" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N112" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N112" s="16" t="inlineStr">
+        <is>
+          <t>INFO ride/pool/driver.transition in the audit writer; WARN command.rejected — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O112" s="16" t="inlineStr"/>
       <c r="P112" s="4">
         <f>","&amp;SUBSTITUTE(F112," ","")&amp;","</f>
@@ -10401,10 +10473,14 @@
       </c>
       <c r="M115" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N115" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N115" s="16" t="inlineStr">
+        <is>
+          <t>Pure fare (feature/zones-fares) and transition checks with unit tests (TC-08) — feature/ride-request</t>
+        </is>
+      </c>
       <c r="O115" s="16" t="inlineStr"/>
       <c r="P115" s="4">
         <f>","&amp;SUBSTITUTE(F115," ","")&amp;","</f>
@@ -12560,11 +12636,19 @@
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J3" s="16" t="inlineStr"/>
-      <c r="K3" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>Ride level in test/rides/cancel.test.ts and test/domain/state-machine.test.ts; pool moves later</t>
+        </is>
+      </c>
+      <c r="K3" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 partial</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -12671,7 +12755,7 @@
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>Role part in test/auth/access.test.ts; ride/pool ownership with those modules</t>
+          <t>Roles in test/auth/access.test.ts; ride ownership in test/rides/read.test.ts and cancel.test.ts; pools later</t>
         </is>
       </c>
       <c r="K5" s="16" t="inlineStr">
@@ -12723,11 +12807,19 @@
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J6" s="16" t="inlineStr"/>
-      <c r="K6" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t>REQUESTED and STARTED in test/rides/cancel.test.ts, policy in test/domain/cancellation.test.ts; MATCHED and DRIVER_ARRIVED later</t>
+        </is>
+      </c>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 partial</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="63" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -12878,11 +12970,19 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J9" s="16" t="inlineStr"/>
-      <c r="K9" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/domain/state-machine.test.ts</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="33" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -13384,11 +13484,19 @@
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J19" s="16" t="inlineStr"/>
-      <c r="K19" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/rides/request.test.ts (no Idempotency-Key: retries rely on the unique index)</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
@@ -13678,11 +13786,19 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J25" s="16" t="inlineStr"/>
-      <c r="K25" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>Read side in test/rides/read.test.ts; the accept part with feature/tesla-pooling</t>
+        </is>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 partial</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="63" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
@@ -14135,11 +14251,19 @@
       </c>
       <c r="I34" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J34" s="16" t="inlineStr"/>
-      <c r="K34" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J34" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/rides/request.test.ts</t>
+        </is>
+      </c>
+      <c r="K34" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="33" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
@@ -14461,11 +14585,19 @@
       </c>
       <c r="I40" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J40" s="16" t="inlineStr"/>
-      <c r="K40" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J40" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/rides/read.test.ts</t>
+        </is>
+      </c>
+      <c r="K40" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="33" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
@@ -15013,7 +15145,7 @@
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>Part 1 (gender optional at sign-up) in test/auth/sign-up.test.ts; option validation with rides</t>
+          <t>Parts 1-3 in test/auth/sign-up.test.ts and test/rides/request.test.ts; passenger side of part 4 in test/rides/read.test.ts; driver pool response later</t>
         </is>
       </c>
       <c r="K51" s="16" t="inlineStr">
@@ -17949,11 +18081,19 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H13" s="16" t="inlineStr"/>
-      <c r="I13" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>97a8fb6 feat(ride) state machines, 97e9a70 feat(audit) — feature/ride-request</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Transition tables shared with the web app; audit writer inside the caller's transaction; WARN log for 409/422</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
@@ -17986,11 +18126,19 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H14" s="16" t="inlineStr"/>
-      <c r="I14" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>0896c40 feat(ride), e32e7bb fix(ride), dcc02ed feat(ride), 75785c0 test(ride) — feature/ride-request</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Create, list, detail, expiry and REQUESTED cancel done; cancelling MATCHED/DRIVER_ARRIVED (seat release, fee) comes with feature/tesla-pooling and feature/driver-flow</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, conventions and tracker with the pooling module
ARCHITECTURE v0.7: GET /api/driver/availability; isCompatible(request, pool, rules) with its fixed check order and how each reason maps to 409 or 422; service names per file for drivers and pools; the §6.2 audit rows; the passenger cancel in MATCHED (pool lock, one re-read) and pools that end while an accept waits for their lock. The conventions guide covers changing neighbours and the join window. Tracker: T-14 and T-15 done, T-16 in progress (README concurrency notes in pre-release); the driver, pool and matching requirements implemented; TC-01, TC-06, TC-16, TC-17, TC-19…TC-24, TC-47…TC-51 passing.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 4 (feature/ride-request): state machines, audit trail, ride requests, expiry, unmatched cancellation</t>
+          <t>2026-09-24 — Phase 5 (feature/tesla-pooling): driver availability and feed, matching, accept with seat locks, matched cancellation, race tests</t>
         </is>
       </c>
     </row>
@@ -3366,10 +3366,14 @@
       </c>
       <c r="M20" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N20" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N20" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/driver/availability returns the Tesla — feature/tesla-pooling; dashboard in feature/driver-ui</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr"/>
       <c r="P20" s="4">
         <f>","&amp;SUBSTITUTE(F20," ","")&amp;","</f>
@@ -3439,10 +3443,14 @@
       </c>
       <c r="M21" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N21" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N21" s="16" t="inlineStr">
+        <is>
+          <t>PUT /api/driver/availability, audited with the zone (TC-22) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O21" s="16" t="inlineStr"/>
       <c r="P21" s="4">
         <f>","&amp;SUBSTITUTE(F21," ","")&amp;","</f>
@@ -3512,10 +3520,14 @@
       </c>
       <c r="M22" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N22" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>409 ACTIVE_POOL_EXISTS for offline or zone change during a trip (TC-22) — feature/tesla-pooling; disabled toggle in feature/driver-ui</t>
+        </is>
+      </c>
       <c r="O22" s="16" t="inlineStr"/>
       <c r="P22" s="4">
         <f>","&amp;SUBSTITUTE(F22," ","")&amp;","</f>
@@ -3585,10 +3597,14 @@
       </c>
       <c r="M23" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N23" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/driver/requests: zone feed, matching filter with an OPEN pool, 409 DRIVER_OFFLINE (TC-23) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O23" s="16" t="inlineStr"/>
       <c r="P23" s="4">
         <f>","&amp;SUBSTITUTE(F23," ","")&amp;","</f>
@@ -3658,10 +3674,14 @@
       </c>
       <c r="M24" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N24" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N24" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/driver/requests/:id/accept re-checks BR-01…05 in one transaction — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O24" s="16" t="inlineStr"/>
       <c r="P24" s="4">
         <f>","&amp;SUBSTITUTE(F24," ","")&amp;","</f>
@@ -3731,10 +3751,14 @@
       </c>
       <c r="M25" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N25" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N25" s="16" t="inlineStr">
+        <is>
+          <t>Pool view (names, seats, status, payment, estimate, badge) returned on accept — feature/tesla-pooling; GET /api/driver/pools and locked fares in feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O25" s="16" t="inlineStr"/>
       <c r="P25" s="4">
         <f>","&amp;SUBSTITUTE(F25," ","")&amp;","</f>
@@ -4315,10 +4339,14 @@
       </c>
       <c r="M33" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N33" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N33" s="16" t="inlineStr">
+        <is>
+          <t>Pool created on first accept, audited null → OPEN — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O33" s="16" t="inlineStr"/>
       <c r="P33" s="4">
         <f>","&amp;SUBSTITUTE(F33," ","")&amp;","</f>
@@ -4388,10 +4416,14 @@
       </c>
       <c r="M34" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N34" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N34" s="16" t="inlineStr">
+        <is>
+          <t>Capacity check under the driver and pool locks plus the DB CHECK; TC-01, TC-06 — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O34" s="16" t="inlineStr"/>
       <c r="P34" s="4">
         <f>","&amp;SUBSTITUTE(F34," ","")&amp;","</f>
@@ -4461,10 +4493,14 @@
       </c>
       <c r="M35" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N35" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N35" s="16" t="inlineStr">
+        <is>
+          <t>isCompatible at accept time; 422 NOT_COMPATIBLE with reason (TC-20) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O35" s="16" t="inlineStr"/>
       <c r="P35" s="4">
         <f>","&amp;SUBSTITUTE(F35," ","")&amp;","</f>
@@ -4534,10 +4570,14 @@
       </c>
       <c r="M36" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N36" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N36" s="16" t="inlineStr">
+        <is>
+          <t>is_private from the first member; TC-19 — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O36" s="16" t="inlineStr"/>
       <c r="P36" s="4">
         <f>","&amp;SUBSTITUTE(F36," ","")&amp;","</f>
@@ -4607,10 +4647,14 @@
       </c>
       <c r="M37" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N37" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N37" s="16" t="inlineStr">
+        <is>
+          <t>409 POOL_NOT_OPEN (TC-21) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O37" s="16" t="inlineStr"/>
       <c r="P37" s="4">
         <f>","&amp;SUBSTITUTE(F37," ","")&amp;","</f>
@@ -4675,15 +4719,19 @@
       </c>
       <c r="L38" s="13" t="inlineStr">
         <is>
-          <t>feature/driver-flow</t>
+          <t>feature/tesla-pooling, feature/driver-flow</t>
         </is>
       </c>
       <c r="M38" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N38" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N38" s="16" t="inlineStr">
+        <is>
+          <t>MATCHED cancel frees seats at once (TC-16) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O38" s="16" t="inlineStr"/>
       <c r="P38" s="4">
         <f>","&amp;SUBSTITUTE(F38," ","")&amp;","</f>
@@ -4748,15 +4796,19 @@
       </c>
       <c r="L39" s="17" t="inlineStr">
         <is>
-          <t>feature/driver-flow</t>
+          <t>feature/tesla-pooling, feature/driver-flow</t>
         </is>
       </c>
       <c r="M39" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N39" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N39" s="16" t="inlineStr">
+        <is>
+          <t>Empty pool cancelled by SYSTEM, ALL_MEMBERS_CANCELLED (TC-16) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O39" s="16" t="inlineStr"/>
       <c r="P39" s="4">
         <f>","&amp;SUBSTITUTE(F39," ","")&amp;","</f>
@@ -4899,12 +4951,12 @@
       </c>
       <c r="M41" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
         <is>
-          <t>pool_members_one_active_membership index tested; accept flow in feature/tesla-pooling — feature/db-schema</t>
+          <t>Partial unique index (feature/db-schema) and ride CAS; Jashim vs Kamal race 20/20 (TC-06) — feature/tesla-pooling</t>
         </is>
       </c>
       <c r="O41" s="16" t="inlineStr"/>
@@ -4976,12 +5028,12 @@
       </c>
       <c r="M42" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N42" s="16" t="inlineStr">
         <is>
-          <t>pool_members table; roster endpoint in feature/driver-flow — feature/db-schema</t>
+          <t>pool_members rows; driver pool view lists members — feature/tesla-pooling</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr"/>
@@ -5053,10 +5105,14 @@
       </c>
       <c r="M43" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N43" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N43" s="16" t="inlineStr">
+        <is>
+          <t>Restriction checked and updated under the pool lock (TC-47, TC-51) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O43" s="16" t="inlineStr">
         <is>
           <t>Added in SRS v0.3</t>
@@ -5125,15 +5181,19 @@
       </c>
       <c r="L44" s="13" t="inlineStr">
         <is>
-          <t>feature/driver-flow</t>
+          <t>feature/tesla-pooling, feature/driver-flow</t>
         </is>
       </c>
       <c r="M44" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N44" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N44" s="16" t="inlineStr">
+        <is>
+          <t>Restriction recalculated on leave (TC-49) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
           <t>Added in SRS v0.3</t>
@@ -6411,10 +6471,14 @@
       </c>
       <c r="M61" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N61" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N61" s="16" t="inlineStr">
+        <is>
+          <t>TC-01, TC-06 — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O61" s="16" t="inlineStr"/>
       <c r="P61" s="4">
         <f>","&amp;SUBSTITUTE(F61," ","")&amp;","</f>
@@ -6484,10 +6548,14 @@
       </c>
       <c r="M62" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N62" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N62" s="16" t="inlineStr">
+        <is>
+          <t>domain/matching.ts; TC-20 — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O62" s="16" t="inlineStr"/>
       <c r="P62" s="4">
         <f>","&amp;SUBSTITUTE(F62," ","")&amp;","</f>
@@ -6557,10 +6625,14 @@
       </c>
       <c r="M63" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N63" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N63" s="16" t="inlineStr">
+        <is>
+          <t>First accept starts a pool in the driver's zone — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O63" s="16" t="inlineStr"/>
       <c r="P63" s="4">
         <f>","&amp;SUBSTITUTE(F63," ","")&amp;","</f>
@@ -6630,10 +6702,14 @@
       </c>
       <c r="M64" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N64" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N64" s="16" t="inlineStr">
+        <is>
+          <t>Driver lock plus pools_one_active_per_driver; TC-19 — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O64" s="16" t="inlineStr"/>
       <c r="P64" s="4">
         <f>","&amp;SUBSTITUTE(F64," ","")&amp;","</f>
@@ -7692,10 +7768,14 @@
       </c>
       <c r="M78" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N78" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N78" s="16" t="inlineStr">
+        <is>
+          <t>domain/pool-restriction.ts + matching; TC-47, TC-48, TC-49, TC-51 — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O78" s="16" t="inlineStr">
         <is>
           <t>Added in SRS v0.3</t>
@@ -8462,10 +8542,14 @@
       </c>
       <c r="M88" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N88" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N88" s="16" t="inlineStr">
+        <is>
+          <t>Last-seat race 20/20 in test/pools/concurrency.test.ts (TC-06) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="O88" s="16" t="inlineStr"/>
       <c r="P88" s="4">
         <f>","&amp;SUBSTITUTE(F88," ","")&amp;","</f>
@@ -8540,7 +8624,7 @@
       </c>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>CAS on status for cancel and expiry, audit in the same transaction — feature/ride-request; accept/pool moves in feature/tesla-pooling</t>
+          <t>CAS for cancel, expiry, match and pool cancel; audit in the same transaction; cancel-vs-accept race (TC-17) — feature/tesla-pooling; arrive/start/drop-off in feature/driver-flow</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr"/>
@@ -8612,12 +8696,12 @@
       </c>
       <c r="M90" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="N90" s="16" t="inlineStr">
         <is>
-          <t>Mechanism designed: ARCHITECTURE.md §7, ADR-0006</t>
+          <t>Driver and pool row locks plus the CHECK, as in ARCHITECTURE §7 — feature/tesla-pooling; README section in pre-release</t>
         </is>
       </c>
       <c r="O90" s="16" t="inlineStr"/>
@@ -9143,12 +9227,12 @@
       </c>
       <c r="M97" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Expiry on read and before every passenger command, plus the 60 s sweep — feature/ride-request; accept check in feature/tesla-pooling</t>
+          <t>Expiry on read, before passenger commands and in the sweep (feature/ride-request); accept refuses expired requests (TC-24) — feature/tesla-pooling</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr"/>
@@ -12587,11 +12671,19 @@
       </c>
       <c r="I2" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J2" s="16" t="inlineStr"/>
-      <c r="K2" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J2" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/accept.test.ts</t>
+        </is>
+      </c>
+      <c r="K2" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="63" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -12812,7 +12904,7 @@
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>REQUESTED and STARTED in test/rides/cancel.test.ts, policy in test/domain/cancellation.test.ts; MATCHED and DRIVER_ARRIVED later</t>
+          <t>REQUESTED, MATCHED (test/pools/leave.test.ts) and STARTED; policy unit test; DRIVER_ARRIVED fee later</t>
         </is>
       </c>
       <c r="K6" s="16" t="inlineStr">
@@ -12864,11 +12956,19 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J7" s="16" t="inlineStr"/>
-      <c r="K7" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/concurrency.test.ts (20 runs each)</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -13386,11 +13486,19 @@
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J17" s="16" t="inlineStr"/>
-      <c r="K17" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/leave.test.ts</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
@@ -13435,11 +13543,19 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J18" s="16" t="inlineStr"/>
-      <c r="K18" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/concurrency.test.ts (20 runs, plus a forced accept-first case)</t>
+        </is>
+      </c>
+      <c r="K18" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -13541,11 +13657,19 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J20" s="16" t="inlineStr"/>
-      <c r="K20" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J20" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/accept.test.ts</t>
+        </is>
+      </c>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -13590,11 +13714,19 @@
       </c>
       <c r="I21" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J21" s="16" t="inlineStr"/>
-      <c r="K21" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/domain/matching.test.ts, apps/api/test/pools/accept.test.ts</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
@@ -13639,11 +13771,19 @@
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J22" s="16" t="inlineStr"/>
-      <c r="K22" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/accept.test.ts</t>
+        </is>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="33" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -13688,11 +13828,19 @@
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J23" s="16" t="inlineStr"/>
-      <c r="K23" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/drivers/availability.test.ts</t>
+        </is>
+      </c>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
@@ -13737,11 +13885,19 @@
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J24" s="16" t="inlineStr"/>
-      <c r="K24" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/drivers/feed.test.ts</t>
+        </is>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -13786,17 +13942,17 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>Read side in test/rides/read.test.ts; the accept part with feature/tesla-pooling</t>
+          <t>apps/api/test/pools/accept.test.ts, apps/api/test/rides/read.test.ts</t>
         </is>
       </c>
       <c r="K25" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 partial</t>
+          <t>2026-09-24 passing (local + Docker)</t>
         </is>
       </c>
     </row>
@@ -14993,11 +15149,19 @@
       </c>
       <c r="I48" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J48" s="16" t="inlineStr"/>
-      <c r="K48" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J48" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/leave.test.ts, apps/api/test/domain/matching.test.ts</t>
+        </is>
+      </c>
+      <c r="K48" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="63" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
@@ -15042,11 +15206,19 @@
       </c>
       <c r="I49" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J49" s="16" t="inlineStr"/>
-      <c r="K49" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J49" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/leave.test.ts, apps/api/test/domain/matching.test.ts</t>
+        </is>
+      </c>
+      <c r="K49" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="33" customHeight="1">
       <c r="A50" s="14" t="inlineStr">
@@ -15091,11 +15263,19 @@
       </c>
       <c r="I50" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J50" s="16" t="inlineStr"/>
-      <c r="K50" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J50" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/leave.test.ts</t>
+        </is>
+      </c>
+      <c r="K50" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="63" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
@@ -15140,17 +15320,17 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>Parts 1-3 in test/auth/sign-up.test.ts and test/rides/request.test.ts; passenger side of part 4 in test/rides/read.test.ts; driver pool response later</t>
+          <t>test/auth/sign-up.test.ts, test/rides/request.test.ts, test/rides/read.test.ts, test/pools/accept.test.ts (no gender in the driver pool view)</t>
         </is>
       </c>
       <c r="K51" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 partial</t>
+          <t>2026-09-24 passing (local + Docker)</t>
         </is>
       </c>
     </row>
@@ -15197,11 +15377,19 @@
       </c>
       <c r="I52" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J52" s="16" t="inlineStr"/>
-      <c r="K52" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J52" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/concurrency.test.ts (20 runs)</t>
+        </is>
+      </c>
+      <c r="K52" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K52"/>
@@ -18136,7 +18324,7 @@
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>Create, list, detail, expiry and REQUESTED cancel done; cancelling MATCHED/DRIVER_ARRIVED (seat release, fee) comes with feature/tesla-pooling and feature/driver-flow</t>
+          <t>Create, list, detail, expiry, REQUESTED and MATCHED cancel done (MATCHED in feature/tesla-pooling); DRIVER_ARRIVED with fee comes with feature/driver-flow</t>
         </is>
       </c>
     </row>
@@ -18171,13 +18359,17 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H15" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>c8637c0 feat(driver) — feature/tesla-pooling</t>
+        </is>
+      </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>Moved from feature/driver-flow: accept needs driver availability first (plan Phase 5)</t>
+          <t>GET/PUT /api/driver/availability (audited); GET /api/driver/requests filtered by the matching rule</t>
         </is>
       </c>
     </row>
@@ -18212,11 +18404,19 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H16" s="16" t="inlineStr"/>
-      <c r="I16" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>6b23f01 feat(pool) matching, 433fb89 feat(pool) accept, cd60b88 feat(pool) leave — feature/tesla-pooling</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>Accept locks driver → pool → ride; CAS on the ride; CHECK as last defence; restriction under the pool lock; MATCHED cancel frees seats</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -18249,11 +18449,19 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H17" s="16" t="inlineStr"/>
-      <c r="I17" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>1e66ae3 test(pool) — feature/tesla-pooling</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>All races pass 20/20 (TC-06, TC-17, TC-51); README concurrency section is written in pre-release</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, conventions and tracker with the driver trip flow
ARCHITECTURE v0.8: driver commands check ownership and then lock driver → pool; §6.4 as built; §6.5 with the one re-read, the restriction update and the fee row; a new §6.6 for the driver cancelling a trip and marking a no-show; pool service names per file. The conventions guide covers the cancellation fee and the no-show wait. Tracker: T-13 and T-17 done; FR-DRV-07/08/11/12, FR-POOL-08, FR-FARE-03/05, BR-07, BR-12, FR-HIST-01 and NFR-CON-02 implemented; TC-02, TC-04, TC-05, TC-09, TC-11, TC-13, TC-15, TC-40 and TC-43 passing.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 5 (feature/tesla-pooling): driver availability and feed, matching, accept with seat locks, matched cancellation, race tests</t>
+          <t>2026-09-24 — Phase 6 (feature/driver-flow): arrive, start with fare lock, drop-off, trip cancel, no-show, cancellation fee</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="N16" s="16" t="inlineStr">
         <is>
-          <t>POST /api/rides/:id/cancel: REQUESTED free, STARTED/terminal 409 — feature/ride-request; MATCHED and DRIVER_ARRIVED (fee) later</t>
+          <t>All states: free in REQUESTED/MATCHED, ৳20 fee in DRIVER_ARRIVED, 409 when started/finished (TC-05) — feature/driver-flow; fee confirmation in feature/passenger-ui</t>
         </is>
       </c>
       <c r="O16" s="16" t="inlineStr"/>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="N25" s="16" t="inlineStr">
         <is>
-          <t>Pool view (names, seats, status, payment, estimate, badge) returned on accept — feature/tesla-pooling; GET /api/driver/pools and locked fares in feature/driver-flow</t>
+          <t>GET /api/driver/pools?scope=active with names, seats, status, payment, estimate/locked fare, badge — feature/driver-flow; screen in feature/driver-ui</t>
         </is>
       </c>
       <c r="O25" s="16" t="inlineStr"/>
@@ -3828,10 +3828,14 @@
       </c>
       <c r="M26" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N26" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N26" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/pools/:id/arrive — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O26" s="16" t="inlineStr"/>
       <c r="P26" s="4">
         <f>","&amp;SUBSTITUTE(F26," ","")&amp;","</f>
@@ -3901,10 +3905,14 @@
       </c>
       <c r="M27" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N27" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N27" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/pools/:id/start; refused with nobody on board — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O27" s="16" t="inlineStr"/>
       <c r="P27" s="4">
         <f>","&amp;SUBSTITUTE(F27," ","")&amp;","</f>
@@ -3974,10 +3982,14 @@
       </c>
       <c r="M28" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N28" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N28" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/pools/:id/members/:rideId/complete, any order, auto-complete, zone update (TC-25) — feature/driver-flow; settlement in feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr"/>
       <c r="P28" s="4">
         <f>","&amp;SUBSTITUTE(F28," ","")&amp;","</f>
@@ -4120,10 +4132,14 @@
       </c>
       <c r="M30" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N30" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N30" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/pools/:id/cancel; members back to REQUESTED free; 409 after start (TC-15) — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O30" s="16" t="inlineStr"/>
       <c r="P30" s="4">
         <f>","&amp;SUBSTITUTE(F30," ","")&amp;","</f>
@@ -4193,10 +4209,14 @@
       </c>
       <c r="M31" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N31" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N31" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/pools/:id/members/:rideId/no-show after NO_SHOW_WAIT_MINUTES, with fee (TC-43) — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O31" s="16" t="inlineStr"/>
       <c r="P31" s="4">
         <f>","&amp;SUBSTITUTE(F31," ","")&amp;","</f>
@@ -4266,10 +4286,14 @@
       </c>
       <c r="M32" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N32" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N32" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/driver/pools?scope=history, own pools only, with totals (TC-40) — feature/driver-flow; screen in feature/driver-ui</t>
+        </is>
+      </c>
       <c r="O32" s="16" t="inlineStr"/>
       <c r="P32" s="4">
         <f>","&amp;SUBSTITUTE(F32," ","")&amp;","</f>
@@ -4878,10 +4902,14 @@
       </c>
       <c r="M40" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N40" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N40" s="16" t="inlineStr">
+        <is>
+          <t>SYSTEM completes the pool after the last drop-off, completed_at set — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O40" s="16" t="inlineStr"/>
       <c r="P40" s="4">
         <f>","&amp;SUBSTITUTE(F40," ","")&amp;","</f>
@@ -5421,10 +5449,14 @@
       </c>
       <c r="M47" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N47" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N47" s="16" t="inlineStr">
+        <is>
+          <t>fares row per on-board member with rate snapshot at start (TC-09, TC-11) — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O47" s="16" t="inlineStr"/>
       <c r="P47" s="4">
         <f>","&amp;SUBSTITUTE(F47," ","")&amp;","</f>
@@ -5499,7 +5531,7 @@
       </c>
       <c r="N48" s="16" t="inlineStr">
         <is>
-          <t>API returns base, distance charge, discount, seats, total (TC-35); views in the UI branches — feature/zones-fares</t>
+          <t>API: estimate and locked breakdowns (rides), locked fares per member and totals (driver) — feature/driver-flow; views in the UI branches</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr"/>
@@ -5571,10 +5603,14 @@
       </c>
       <c r="M49" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N49" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N49" s="16" t="inlineStr">
+        <is>
+          <t>CANCELLATION_FEE charge row on passenger cancel after arrival and on no-show — feature/driver-flow</t>
+        </is>
+      </c>
       <c r="O49" s="16" t="inlineStr"/>
       <c r="P49" s="4">
         <f>","&amp;SUBSTITUTE(F49," ","")&amp;","</f>
@@ -6163,12 +6199,12 @@
       </c>
       <c r="M57" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N57" s="16" t="inlineStr">
         <is>
-          <t>recordTransition in the same transaction: ride create, cancel, expiry — feature/ride-request; pool and driver transitions follow</t>
+          <t>Every ride, pool and driver transition audited in its transaction — feature/driver-flow</t>
         </is>
       </c>
       <c r="O57" s="16" t="inlineStr"/>
@@ -7010,12 +7046,12 @@
       </c>
       <c r="M68" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N68" s="16" t="inlineStr">
         <is>
-          <t>domain/cancellation.ts policy (FREE/FEE/FORBIDDEN); fee charging in feature/driver-flow — feature/ride-request</t>
+          <t>cancellationPolicy (feature/ride-request); fee recorded after arrival and on no-show; refused once started — feature/driver-flow</t>
         </is>
       </c>
       <c r="O68" s="16" t="inlineStr"/>
@@ -7318,12 +7354,12 @@
       </c>
       <c r="M72" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N72" s="16" t="inlineStr">
         <is>
-          <t>computeFare takes the pooled flag (TC-10: 2 seats of 1 passenger not pooled); locking at start in feature/driver-flow — feature/zones-fares</t>
+          <t>pooled = two or more members start together; fare and rates stored at start (TC-09) — feature/driver-flow</t>
         </is>
       </c>
       <c r="O72" s="16" t="inlineStr"/>
@@ -8008,7 +8044,7 @@
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Role guards (feature/passenger-auth); rides scoped to their owner, 404 for others (TC-04 part) — feature/ride-request</t>
+          <t>Rides scoped to their passenger; driver commands and pool lists scoped to the owning driver, 404 otherwise (TC-04) — feature/driver-flow; wallet later</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr"/>
@@ -8619,12 +8655,12 @@
       </c>
       <c r="M89" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>CAS for cancel, expiry, match and pool cancel; audit in the same transaction; cancel-vs-accept race (TC-17) — feature/tesla-pooling; arrive/start/drop-off in feature/driver-flow</t>
+          <t>Every transition is a CAS inside a transaction with its side effects and audit row (TC-02, TC-17) — feature/driver-flow</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr"/>
@@ -12728,17 +12764,17 @@
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J3" s="16" t="inlineStr">
         <is>
-          <t>Ride level in test/rides/cancel.test.ts and test/domain/state-machine.test.ts; pool moves later</t>
+          <t>apps/api/test/pools/cancel-trip.test.ts, trip.test.ts, journey.test.ts, rides/cancel.test.ts, domain/state-machine.test.ts</t>
         </is>
       </c>
       <c r="K3" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 partial</t>
+          <t>2026-09-24 passing (local + Docker)</t>
         </is>
       </c>
     </row>
@@ -12842,17 +12878,17 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>Roles in test/auth/access.test.ts; ride ownership in test/rides/read.test.ts and cancel.test.ts; pools later</t>
+          <t>apps/api/test/pools/cancel-trip.test.ts, rides/read.test.ts, rides/cancel.test.ts, auth/access.test.ts</t>
         </is>
       </c>
       <c r="K5" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 partial</t>
+          <t>2026-09-24 passing (local + Docker)</t>
         </is>
       </c>
     </row>
@@ -12899,17 +12935,17 @@
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>REQUESTED, MATCHED (test/pools/leave.test.ts) and STARTED; policy unit test; DRIVER_ARRIVED fee later</t>
+          <t>apps/api/test/rides/cancel.test.ts, pools/leave.test.ts, pools/cancel-trip.test.ts, domain/cancellation.test.ts</t>
         </is>
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 partial</t>
+          <t>2026-09-24 passing (local + Docker)</t>
         </is>
       </c>
     </row>
@@ -13127,11 +13163,19 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J10" s="16" t="inlineStr"/>
-      <c r="K10" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/trip.test.ts</t>
+        </is>
+      </c>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -13233,11 +13277,19 @@
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J12" s="16" t="inlineStr"/>
-      <c r="K12" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/trip.test.ts</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -13339,11 +13391,19 @@
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J14" s="16" t="inlineStr"/>
-      <c r="K14" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/journey.test.ts, rides/read.test.ts</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
@@ -13437,11 +13497,19 @@
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J16" s="16" t="inlineStr"/>
-      <c r="K16" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/cancel-trip.test.ts</t>
+        </is>
+      </c>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -13999,11 +14067,19 @@
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J26" s="16" t="inlineStr"/>
-      <c r="K26" s="16" t="inlineStr"/>
+          <t>Written</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>Statuses, drop-off order, auto-complete and zone in apps/api/test/pools/journey.test.ts; payments with feature/teslapay-wallet</t>
+        </is>
+      </c>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 partial</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
@@ -14798,11 +14874,19 @@
       </c>
       <c r="I41" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J41" s="16" t="inlineStr"/>
-      <c r="K41" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J41" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/journey.test.ts, drivers/availability.test.ts</t>
+        </is>
+      </c>
+      <c r="K41" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
@@ -14945,11 +15029,19 @@
       </c>
       <c r="I44" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J44" s="16" t="inlineStr"/>
-      <c r="K44" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J44" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/pools/cancel-trip.test.ts</t>
+        </is>
+      </c>
+      <c r="K44" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
@@ -18314,7 +18406,7 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
@@ -18324,7 +18416,7 @@
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>Create, list, detail, expiry, REQUESTED and MATCHED cancel done (MATCHED in feature/tesla-pooling); DRIVER_ARRIVED with fee comes with feature/driver-flow</t>
+          <t>Create, list, detail, expiry; cancel in REQUESTED, MATCHED (feature/tesla-pooling) and DRIVER_ARRIVED with the fee (feature/driver-flow)</t>
         </is>
       </c>
     </row>
@@ -18494,11 +18586,19 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H18" s="16" t="inlineStr"/>
-      <c r="I18" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>f51318f, 3768aad, 12762d8 feat(driver); e03dc7d test(driver) — feature/driver-flow</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Arrive, start with fare lock, drop-off with auto-complete and zone update, cancel trip, no-show, GET /api/driver/pools</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, ERD, conventions and tracker with the wallet module
ARCHITECTURE v0.9: the wallet and settlement services, cash collection as a pools route, the cash fall-back and PAYMENT audit rows in §6.4, and the unreachable-database codes mapped to 503. ERD v0.4: PAYMENT in audit_entity with its migration, and the payment rules as built. The conventions guide covers the top-up limits and moving money only through the wallet service. Tracker: T-18 done; FR-PAY-03…06, FR-DRV-09/10, FR-HIST-04, BR-15…17, NFR-CON-05, NFR-REL-03 and NFR-SEC-03 implemented; TC-14, TC-25…TC-30 and TC-42 passing.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 6 (feature/driver-flow): arrive, start with fare lock, drop-off, trip cancel, no-show, cancellation fee</t>
+          <t>2026-09-24 — Phase 7 (feature/teslapay-wallet): wallet, top-up, settlement, cash collection, fees, E1–E5 end to end</t>
         </is>
       </c>
     </row>
@@ -3982,12 +3982,12 @@
       </c>
       <c r="M28" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N28" s="16" t="inlineStr">
         <is>
-          <t>POST /api/pools/:id/members/:rideId/complete, any order, auto-complete, zone update (TC-25) — feature/driver-flow; settlement in feature/teslapay-wallet</t>
+          <t>Drop-off in any order with settlement in the same transaction, auto-complete, zone update (feature/driver-flow, feature/teslapay-wallet)</t>
         </is>
       </c>
       <c r="O28" s="16" t="inlineStr"/>
@@ -4059,10 +4059,14 @@
       </c>
       <c r="M29" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N29" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N29" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/pools/:id/members/:rideId/cash-collected, once, owner only, PAYMENT audit row (TC-27) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O29" s="16" t="inlineStr"/>
       <c r="P29" s="4">
         <f>","&amp;SUBSTITUTE(F29," ","")&amp;","</f>
@@ -5757,10 +5761,14 @@
       </c>
       <c r="M51" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N51" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N51" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/wallet and /api/wallet/transactions (newest first, paged) — feature/teslapay-wallet; screen in feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O51" s="16" t="inlineStr"/>
       <c r="P51" s="4">
         <f>","&amp;SUBSTITUTE(F51," ","")&amp;","</f>
@@ -5830,10 +5838,14 @@
       </c>
       <c r="M52" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N52" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N52" s="16" t="inlineStr">
+        <is>
+          <t>POST /api/wallet/topup ৳50–৳5,000, TOPUP ledger entry (TC-29) — feature/teslapay-wallet; 'simulated' label in feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O52" s="16" t="inlineStr"/>
       <c r="P52" s="4">
         <f>","&amp;SUBSTITUTE(F52," ","")&amp;","</f>
@@ -5903,10 +5915,14 @@
       </c>
       <c r="M53" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N53" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N53" s="16" t="inlineStr">
+        <is>
+          <t>TeslaPay debit at drop-off with RIDE_PAYMENT entry, PAID (TC-26) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O53" s="16" t="inlineStr"/>
       <c r="P53" s="4">
         <f>","&amp;SUBSTITUTE(F53," ","")&amp;","</f>
@@ -5976,10 +5992,14 @@
       </c>
       <c r="M54" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N54" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N54" s="16" t="inlineStr">
+        <is>
+          <t>Cash rides PENDING_CASH until collected (TC-27) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O54" s="16" t="inlineStr"/>
       <c r="P54" s="4">
         <f>","&amp;SUBSTITUTE(F54," ","")&amp;","</f>
@@ -6049,10 +6069,14 @@
       </c>
       <c r="M55" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N55" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N55" s="16" t="inlineStr">
+        <is>
+          <t>Fee debited from TeslaPay; UNPAID for cash or a short balance (TC-14) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O55" s="16" t="inlineStr"/>
       <c r="P55" s="4">
         <f>","&amp;SUBSTITUTE(F55," ","")&amp;","</f>
@@ -6122,12 +6146,12 @@
       </c>
       <c r="M56" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N56" s="16" t="inlineStr">
         <is>
-          <t>wallets_balance_check + append-only ledger tested; settlement in feature/teslapay-wallet — feature/db-schema</t>
+          <t>CHECK balance &gt;= 0; one ledger entry per change; balance = Σ ledger checked after every wallet test — feature/teslapay-wallet</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr"/>
@@ -6430,12 +6454,12 @@
       </c>
       <c r="M60" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N60" s="16" t="inlineStr">
         <is>
-          <t>Ride, timeline and fare rows readable per ride — feature/ride-request; full E1 reconstruction after feature/teslapay-wallet</t>
+          <t>E1 reconstructed from ride, pool, fare, payment, ledger and audit rows (TC-30, test/e2e/scenarios.test.ts) — feature/teslapay-wallet</t>
         </is>
       </c>
       <c r="O60" s="16" t="inlineStr"/>
@@ -7585,10 +7609,14 @@
       </c>
       <c r="M75" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N75" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N75" s="16" t="inlineStr">
+        <is>
+          <t>Debit in the drop-off transaction; A-14 fall-back to PENDING_CASH (TC-26) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O75" s="16" t="inlineStr"/>
       <c r="P75" s="4">
         <f>","&amp;SUBSTITUTE(F75," ","")&amp;","</f>
@@ -7658,10 +7686,14 @@
       </c>
       <c r="M76" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N76" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N76" s="16" t="inlineStr">
+        <is>
+          <t>PENDING_CASH → PAID when collected (TC-27) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O76" s="16" t="inlineStr"/>
       <c r="P76" s="4">
         <f>","&amp;SUBSTITUTE(F76," ","")&amp;","</f>
@@ -7731,10 +7763,14 @@
       </c>
       <c r="M77" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N77" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N77" s="16" t="inlineStr">
+        <is>
+          <t>topUpSchema limits, credited at once (TC-29) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O77" s="16" t="inlineStr"/>
       <c r="P77" s="4">
         <f>","&amp;SUBSTITUTE(F77," ","")&amp;","</f>
@@ -8039,12 +8075,12 @@
       </c>
       <c r="M81" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Rides scoped to their passenger; driver commands and pool lists scoped to the owning driver, 404 otherwise (TC-04) — feature/driver-flow; wallet later</t>
+          <t>Rides, pools, driver lists and wallets are all scoped to their owner; others get 404 or 403 (TC-04) — feature/teslapay-wallet</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr"/>
@@ -8886,10 +8922,14 @@
       </c>
       <c r="M92" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N92" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N92" s="16" t="inlineStr">
+        <is>
+          <t>Wallet row locked last; guarded debit; ledger entry in the same transaction; concurrent top-ups and top-up vs fare keep balance = Σ ledger — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O92" s="16" t="inlineStr"/>
       <c r="P92" s="4">
         <f>","&amp;SUBSTITUTE(F92," ","")&amp;","</f>
@@ -9190,10 +9230,14 @@
       </c>
       <c r="M96" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N96" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N96" s="16" t="inlineStr">
+        <is>
+          <t>P1001/P1002/P1017 → 503, recovers without restart (TC-42 manual, test/db/errors.test.ts) — feature/teslapay-wallet</t>
+        </is>
+      </c>
       <c r="O96" s="16" t="inlineStr"/>
       <c r="P96" s="4">
         <f>","&amp;SUBSTITUTE(F96," ","")&amp;","</f>
@@ -13448,11 +13492,19 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="inlineStr"/>
-      <c r="K15" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/wallet/fees.test.ts</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
@@ -14067,17 +14119,17 @@
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>Statuses, drop-off order, auto-complete and zone in apps/api/test/pools/journey.test.ts; payments with feature/teslapay-wallet</t>
+          <t>apps/api/test/e2e/scenarios.test.ts (E1), apps/api/test/pools/journey.test.ts</t>
         </is>
       </c>
       <c r="K26" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 partial</t>
+          <t>2026-09-24 passing (local + Docker)</t>
         </is>
       </c>
     </row>
@@ -14124,11 +14176,19 @@
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J27" s="16" t="inlineStr"/>
-      <c r="K27" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/wallet/settlement.test.ts</t>
+        </is>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
@@ -14173,11 +14233,19 @@
       </c>
       <c r="I28" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J28" s="16" t="inlineStr"/>
-      <c r="K28" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/wallet/settlement.test.ts, apps/api/test/e2e/scenarios.test.ts</t>
+        </is>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="33" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -14222,11 +14290,19 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J29" s="16" t="inlineStr"/>
-      <c r="K29" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J29" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/wallet/wallet.test.ts</t>
+        </is>
+      </c>
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="33" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
@@ -14271,11 +14347,19 @@
       </c>
       <c r="I30" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J30" s="16" t="inlineStr"/>
-      <c r="K30" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/wallet/wallet.test.ts</t>
+        </is>
+      </c>
+      <c r="K30" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
@@ -14320,11 +14404,19 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J31" s="16" t="inlineStr"/>
-      <c r="K31" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>apps/api/test/e2e/scenarios.test.ts (E1 audit rows)</t>
+        </is>
+      </c>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (local + Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
@@ -14980,11 +15072,19 @@
       </c>
       <c r="I43" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J43" s="16" t="inlineStr"/>
-      <c r="K43" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J43" s="16" t="inlineStr">
+        <is>
+          <t>Manual: docker compose stop db → wallet 503, health 503; start db → 200 without API restart. Mapping in apps/api/test/db/errors.test.ts</t>
+        </is>
+      </c>
+      <c r="K43" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-24 passing (manual, Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="33" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
@@ -18631,11 +18731,19 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H19" s="16" t="inlineStr"/>
-      <c r="I19" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>a2cba32, a78753d, fc683ad feat(wallet); d2b8f2e test(wallet); e840ff2 test(e2e); cd02042 fix(db) — feature/teslapay-wallet</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Wallet, statement, top-up; settlement at drop-off with cash fall-back; cash collected; fees charged; E1–E5 end to end</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs(adr): add neo-brutalist UI style decision
ADR-0013 records the web app's visual style: 3 px black borders, hard 4px 4px 0 #000 shadows, flat accents with black text (yellow actions, pink fees, cyan info, lime success, red errors) on #FFFDF5, Archivo Black headings and Space Grotesk body text, and status badges that always carry a text label. The tokens live in one CSS file and pages use only the components/ui kit, so the look changes in one place. It compares minimal Tailwind and a component library, and states the accessibility rules that keep contrast and focus visible (NFR-USA-05).

SRS v0.4 adds decision D-25 (no requirement changed); ARCHITECTURE v0.10 §10 describes the style and now implements SRS v0.4; the ADR index lists ADR-0013; the tracker has the D-25 row and the new SRS version.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -722,7 +722,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>0.3 (Draft for review) — see SRS revision history</t>
+          <t>0.4 (Draft for review) — see SRS revision history</t>
         </is>
       </c>
     </row>
@@ -15621,7 +15621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17609,49 +17609,57 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="33" customHeight="1">
+    <row r="47" ht="48" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>D-25</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>PRD inconsistency</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>The PRD mandates a master branch, but the repository was initialised with main.</t>
+          <t>The web app uses a neo-brutalist visual style: 3 px black borders, hard offset shadows, flat bold colours with black text, defined once as tokens and a small component kit (ADR-0013).</t>
         </is>
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>Create master and use it as the integration branch (DR-01).</t>
-        </is>
-      </c>
-      <c r="E47" s="17" t="n"/>
+          <t>High contrast and visible focus by design (NFR-USA-05), a recognisable look without a library dependency, one place to change the look.</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Minimal Tailwind with no defined style; a component library (MUI, shadcn/ui)</t>
+        </is>
+      </c>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>DR-01</t>
+          <t>NFR-USA-01, NFR-USA-02, NFR-USA-05, NFR-USA-06</t>
         </is>
       </c>
       <c r="G47" s="15" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="I47" s="16" t="n"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I47" s="16" t="inlineStr">
+        <is>
+          <t>Requested by product owner</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="33" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>P-01</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -17661,18 +17669,18 @@
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>PRD §18 refers to "the concurrency problem in Section 14". It is actually in §12.</t>
+          <t>The PRD mandates a master branch, but the repository was initialised with main.</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Treated as §12.</t>
+          <t>Create master and use it as the integration branch (DR-01).</t>
         </is>
       </c>
       <c r="E48" s="13" t="n"/>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>NFR-CON-01</t>
+          <t>DR-01</t>
         </is>
       </c>
       <c r="G48" s="15" t="inlineStr">
@@ -17690,7 +17698,7 @@
     <row r="49" ht="33" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>P-02</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -17700,18 +17708,18 @@
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>The PRD lifecycle mixes passenger-level and trip-level states.</t>
+          <t>PRD §18 refers to "the concurrency problem in Section 14". It is actually in §12.</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>Split into two state machines (D-12).</t>
+          <t>Treated as §12.</t>
         </is>
       </c>
       <c r="E49" s="17" t="n"/>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>§5</t>
+          <t>NFR-CON-01</t>
         </is>
       </c>
       <c r="G49" s="15" t="inlineStr">
@@ -17729,28 +17737,28 @@
     <row r="50" ht="33" customHeight="1">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>OI-01</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Open issue</t>
+          <t>PRD inconsistency</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Choose the backend framework, ORM, auth mechanism, test framework, styling and hosting, each justified per DC-07.</t>
+          <t>The PRD lifecycle mixes passenger-level and trip-level states.</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Resolved 2026-09-24: D-14…D-22, ADR-0001…0012</t>
+          <t>Split into two state machines (D-12).</t>
         </is>
       </c>
       <c r="E50" s="13" t="n"/>
       <c r="F50" s="13" t="inlineStr">
         <is>
-          <t>DC-07, DR-07</t>
+          <t>§5</t>
         </is>
       </c>
       <c r="G50" s="15" t="inlineStr">
@@ -17760,7 +17768,7 @@
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="I50" s="16" t="n"/>
@@ -17768,7 +17776,7 @@
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>OI-02</t>
+          <t>OI-01</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -17778,18 +17786,18 @@
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>Choose the concrete concurrency mechanism (pessimistic SELECT … FOR UPDATE versus a conditional update guarded by CHECK) and document it.</t>
+          <t>Choose the backend framework, ORM, auth mechanism, test framework, styling and hosting, each justified per DC-07.</t>
         </is>
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
-          <t>Resolved 2026-09-24: row locks + CAS + constraints in layers (D-18, ADR-0006)</t>
+          <t>Resolved 2026-09-24: D-14…D-22, ADR-0001…0012</t>
         </is>
       </c>
       <c r="E51" s="17" t="n"/>
       <c r="F51" s="17" t="inlineStr">
         <is>
-          <t>NFR-CON-03</t>
+          <t>DC-07, DR-07</t>
         </is>
       </c>
       <c r="G51" s="15" t="inlineStr">
@@ -17807,7 +17815,7 @@
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>OI-03</t>
+          <t>OI-02</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
@@ -17817,31 +17825,70 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Decide whether the request-expiry sweeper runs as an in-process interval or lazily on read (NFR-REL-04 requires lazy correctness either way).</t>
+          <t>Choose the concrete concurrency mechanism (pessimistic SELECT … FOR UPDATE versus a conditional update guarded by CHECK) and document it.</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Resolved 2026-09-24: expiry checked in accept CAS, plus 60 s in-process sweeper (D-18)</t>
+          <t>Resolved 2026-09-24: row locks + CAS + constraints in layers (D-18, ADR-0006)</t>
         </is>
       </c>
       <c r="E52" s="13" t="n"/>
       <c r="F52" s="13" t="inlineStr">
         <is>
+          <t>NFR-CON-03</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="H52" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I52" s="16" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>OI-03</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>Open issue</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Decide whether the request-expiry sweeper runs as an in-process interval or lazily on read (NFR-REL-04 requires lazy correctness either way).</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Resolved 2026-09-24: expiry checked in accept CAS, plus 60 s in-process sweeper (D-18)</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="n"/>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
           <t>NFR-REL-04</t>
         </is>
       </c>
-      <c r="G52" s="15" t="inlineStr">
+      <c r="G53" s="15" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
       </c>
-      <c r="H52" s="14" t="inlineStr">
+      <c r="H53" s="9" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="I52" s="16" t="n"/>
+      <c r="I53" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I52"/>

</xml_diff>

<commit_message>
docs: sync architecture, conventions and tracker with the passenger UI
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 — Phase 7 (feature/teslapay-wallet): wallet, top-up, settlement, cash collection, fees, E1–E5 end to end</t>
+          <t>2026-09-25 — Phase 8 (feature/passenger-ui): UI kit, auth pages, ride request, live tracker, history, ride detail, TeslaPay wallet</t>
         </is>
       </c>
     </row>
@@ -2304,12 +2304,12 @@
       </c>
       <c r="M6" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N6" s="16" t="inlineStr">
         <is>
-          <t>API role guards done (test/auth/access.test.ts); web routing in feature/passenger-ui — feature/passenger-auth</t>
+          <t>API role guards (test/auth/access.test.ts); web group layouts redirect by role via lib/server-session.ts — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr"/>
@@ -2596,12 +2596,12 @@
       </c>
       <c r="M10" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N10" s="16" t="inlineStr">
         <is>
-          <t>POST /api/fares/estimate returns solo and pooled (TC-35); form in feature/passenger-ui — feature/zones-fares</t>
+          <t>POST /api/fares/estimate (TC-35); /ride shows solo and shared prices as the trip is chosen — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr"/>
@@ -2904,12 +2904,12 @@
       </c>
       <c r="M14" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N14" s="16" t="inlineStr">
         <is>
-          <t>GET /api/rides?scope=active and /:id with driver, Tesla, co-rider count, badge — feature/ride-request; screen in feature/passenger-ui</t>
+          <t>Ride tracker: status stepper, driver, Tesla and plate, co-rider count, restriction badge — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O14" s="16" t="inlineStr"/>
@@ -2981,10 +2981,14 @@
       </c>
       <c r="M15" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N15" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N15" s="16" t="inlineStr">
+        <is>
+          <t>useActiveRide/useRide refresh every 4 s while active, no reload needed — feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O15" s="16" t="inlineStr"/>
       <c r="P15" s="4">
         <f>","&amp;SUBSTITUTE(F15," ","")&amp;","</f>
@@ -3054,12 +3058,12 @@
       </c>
       <c r="M16" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N16" s="16" t="inlineStr">
         <is>
-          <t>All states: free in REQUESTED/MATCHED, ৳20 fee in DRIVER_ARRIVED, 409 when started/finished (TC-05) — feature/driver-flow; fee confirmation in feature/passenger-ui</t>
+          <t>API rules (TC-05, feature/driver-flow); cancel dialog states free or the ৳20 fee before confirming — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O16" s="16" t="inlineStr"/>
@@ -3131,12 +3135,12 @@
       </c>
       <c r="M17" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N17" s="16" t="inlineStr">
         <is>
-          <t>GET /api/rides?scope=history, newest first, cursor paging (TC-39) — feature/ride-request; screen in feature/passenger-ui</t>
+          <t>GET /api/rides?scope=history (TC-39); /rides paged list with Show more — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O17" s="16" t="inlineStr"/>
@@ -3208,12 +3212,12 @@
       </c>
       <c r="M18" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N18" s="16" t="inlineStr">
         <is>
-          <t>GET /api/rides/:id timeline from status_history — feature/ride-request; screen in feature/passenger-ui</t>
+          <t>GET /api/rides/:id; /rides/[id] timeline from status_history and fare breakdown — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O18" s="16" t="inlineStr"/>
@@ -3285,12 +3289,12 @@
       </c>
       <c r="M19" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N19" s="16" t="inlineStr">
         <is>
-          <t>Option validation (TC-50 parts 2-3) — feature/ride-request; matching in feature/tesla-pooling, badge in the UI</t>
+          <t>Validation (TC-50), matching (feature/tesla-pooling); same-gender toggle and Women-only/Men-only badge — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O19" s="16" t="inlineStr">
@@ -5535,7 +5539,7 @@
       </c>
       <c r="N48" s="16" t="inlineStr">
         <is>
-          <t>API: estimate and locked breakdowns (rides), locked fares per member and totals (driver) — feature/driver-flow; views in the UI branches</t>
+          <t>Passenger views show the estimate and locked breakdowns (FareBreakdown) — feature/passenger-ui; driver views in feature/driver-ui</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr"/>
@@ -5684,12 +5688,12 @@
       </c>
       <c r="M50" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N50" s="16" t="inlineStr">
         <is>
-          <t>BIGINT paisa columns (feature/db-schema); integer-only fare arithmetic in domain/money.ts (feature/zones-fares); display formatting in the UI</t>
+          <t>BIGINT paisa columns (feature/db-schema); integer arithmetic (domain/money.ts); display only via formatPaisa / MoneyText — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr"/>
@@ -5761,12 +5765,12 @@
       </c>
       <c r="M51" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N51" s="16" t="inlineStr">
         <is>
-          <t>GET /api/wallet and /api/wallet/transactions (newest first, paged) — feature/teslapay-wallet; screen in feature/passenger-ui</t>
+          <t>GET /api/wallet, /api/wallet/transactions; /wallet balance and paged statement — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O51" s="16" t="inlineStr"/>
@@ -5838,12 +5842,12 @@
       </c>
       <c r="M52" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N52" s="16" t="inlineStr">
         <is>
-          <t>POST /api/wallet/topup ৳50–৳5,000, TOPUP ledger entry (TC-29) — feature/teslapay-wallet; 'simulated' label in feature/passenger-ui</t>
+          <t>POST /api/wallet/topup (TC-29); /wallet top-up in taka, labelled simulated — feature/passenger-ui</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr"/>
@@ -9534,10 +9538,14 @@
       </c>
       <c r="M100" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N100" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N100" s="16" t="inlineStr">
+        <is>
+          <t>refetchInterval 4 s while active, stops when terminal, paused while the tab is hidden — feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O100" s="16" t="inlineStr"/>
       <c r="P100" s="4">
         <f>","&amp;SUBSTITUTE(F100," ","")&amp;","</f>
@@ -9607,10 +9615,14 @@
       </c>
       <c r="M101" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N101" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N101" s="16" t="inlineStr">
+        <is>
+          <t>LoadingState, EmptyState, ErrorState with retry on every query-driven passenger view — feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O101" s="16" t="inlineStr"/>
       <c r="P101" s="4">
         <f>","&amp;SUBSTITUTE(F101," ","")&amp;","</f>
@@ -9680,10 +9692,14 @@
       </c>
       <c r="M102" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N102" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N102" s="16" t="inlineStr">
+        <is>
+          <t>lib/labels.ts human labels; StatusStepper and ride timeline — feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O102" s="16" t="inlineStr"/>
       <c r="P102" s="4">
         <f>","&amp;SUBSTITUTE(F102," ","")&amp;","</f>
@@ -9753,10 +9769,14 @@
       </c>
       <c r="M103" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N103" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N103" s="16" t="inlineStr">
+        <is>
+          <t>Cancel shown only when the API allows it — feature/passenger-ui; driver actions in feature/driver-ui</t>
+        </is>
+      </c>
       <c r="O103" s="16" t="inlineStr"/>
       <c r="P103" s="4">
         <f>","&amp;SUBSTITUTE(F103," ","")&amp;","</f>
@@ -9826,10 +9846,14 @@
       </c>
       <c r="M104" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N104" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N104" s="16" t="inlineStr">
+        <is>
+          <t>MoneyText/formatPaisa ৳ with two decimals; breakdown on the tracker and ride detail — feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O104" s="16" t="inlineStr"/>
       <c r="P104" s="4">
         <f>","&amp;SUBSTITUTE(F104," ","")&amp;","</f>
@@ -9899,10 +9923,14 @@
       </c>
       <c r="M105" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N105" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N105" s="16" t="inlineStr">
+        <is>
+          <t>Labelled controls, thick focus outlines, black-on-accent contrast (ADR-0013), 360 px layout — feature/passenger-ui</t>
+        </is>
+      </c>
       <c r="O105" s="16" t="inlineStr"/>
       <c r="P105" s="4">
         <f>","&amp;SUBSTITUTE(F105," ","")&amp;","</f>
@@ -9972,10 +10000,14 @@
       </c>
       <c r="M106" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N106" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N106" s="16" t="inlineStr">
+        <is>
+          <t>Cancel-ride ConfirmDialog states the fee — feature/passenger-ui; cancel pool in feature/driver-ui</t>
+        </is>
+      </c>
       <c r="O106" s="16" t="inlineStr"/>
       <c r="P106" s="4">
         <f>","&amp;SUBSTITUTE(F106," ","")&amp;","</f>
@@ -18823,11 +18855,19 @@
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H20" s="16" t="inlineStr"/>
-      <c r="I20" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>4146169 docs(adr); 8d69a7d, e044886, 79c3d62 feat(web) — feature/passenger-ui</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>ADR-0013 and the neo-brutalist UI kit; API client and query setup; sign-in, sign-up, role routing, shared loading/empty/error states</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -18860,11 +18900,19 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H21" s="16" t="inlineStr"/>
-      <c r="I21" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>426e79b feat(web); 7c08021 feat(ride); a89a16b feat(web) — feature/passenger-ui</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Request form with live solo/shared estimate and same-gender option; live tracker polling every 4 s; cancel dialog stating the fee (API now reports whether and at what cost a ride can be cancelled)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
@@ -18897,11 +18945,19 @@
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H22" s="16" t="inlineStr"/>
-      <c r="I22" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>feat(web): add ride history, ride detail and wallet pages — feature/passenger-ui</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Paged ride history; ride detail with timeline and fare breakdown; TeslaPay balance, simulated top-up in taka, paged statement</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync architecture, conventions and tracker with the driver UI
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25 — Phase 8 (feature/passenger-ui): UI kit, auth pages, ride request, live tracker, history, ride detail, TeslaPay wallet</t>
+          <t>2026-09-25 — Phase 9 (feature/driver-ui): driver dashboard, request feed, active trip management, trip history</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="M20" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N20" s="16" t="inlineStr">
         <is>
-          <t>GET /api/driver/availability returns the Tesla — feature/tesla-pooling; dashboard in feature/driver-ui</t>
+          <t>GET /api/driver/availability (feature/tesla-pooling); /driver shows the Tesla, plate, seats and status — feature/driver-ui</t>
         </is>
       </c>
       <c r="O20" s="16" t="inlineStr"/>
@@ -3524,12 +3524,12 @@
       </c>
       <c r="M22" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N22" s="16" t="inlineStr">
         <is>
-          <t>409 ACTIVE_POOL_EXISTS for offline or zone change during a trip (TC-22) — feature/tesla-pooling; disabled toggle in feature/driver-ui</t>
+          <t>409 ACTIVE_POOL_EXISTS (TC-22, feature/tesla-pooling); zone and online toggle locked with the reason during a trip — feature/driver-ui</t>
         </is>
       </c>
       <c r="O22" s="16" t="inlineStr"/>
@@ -3755,12 +3755,12 @@
       </c>
       <c r="M25" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N25" s="16" t="inlineStr">
         <is>
-          <t>GET /api/driver/pools?scope=active with names, seats, status, payment, estimate/locked fare, badge — feature/driver-flow; screen in feature/driver-ui</t>
+          <t>GET /api/driver/pools?scope=active (feature/driver-flow); /driver/pool shows names, seats, status, payment, estimate or fixed fare, badges — feature/driver-ui</t>
         </is>
       </c>
       <c r="O25" s="16" t="inlineStr"/>
@@ -4294,12 +4294,12 @@
       </c>
       <c r="M32" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N32" s="16" t="inlineStr">
         <is>
-          <t>GET /api/driver/pools?scope=history, own pools only, with totals (TC-40) — feature/driver-flow; screen in feature/driver-ui</t>
+          <t>GET /api/driver/pools?scope=history (TC-40, feature/driver-flow); /driver/history paged with fares and payments — feature/driver-ui</t>
         </is>
       </c>
       <c r="O32" s="16" t="inlineStr"/>
@@ -5534,12 +5534,12 @@
       </c>
       <c r="M48" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N48" s="16" t="inlineStr">
         <is>
-          <t>Passenger views show the estimate and locked breakdowns (FareBreakdown) — feature/passenger-ui; driver views in feature/driver-ui</t>
+          <t>Passenger breakdowns (feature/passenger-ui); per-passenger and trip totals on the driver screens — feature/driver-ui</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr"/>
@@ -9769,12 +9769,12 @@
       </c>
       <c r="M103" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Cancel shown only when the API allows it — feature/passenger-ui; driver actions in feature/driver-ui</t>
+          <t>Passenger Cancel from the API's cancellation (feature/passenger-ui); driver buttons from the shared transition tables via lib/driver-moves.ts — feature/driver-ui</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr"/>
@@ -10000,12 +10000,12 @@
       </c>
       <c r="M106" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N106" s="16" t="inlineStr">
         <is>
-          <t>Cancel-ride ConfirmDialog states the fee — feature/passenger-ui; cancel pool in feature/driver-ui</t>
+          <t>Cancel ride states the fee (feature/passenger-ui); Cancel trip and No-show confirm and say who is charged — feature/driver-ui</t>
         </is>
       </c>
       <c r="O106" s="16" t="inlineStr"/>
@@ -18990,11 +18990,19 @@
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H23" s="16" t="inlineStr"/>
-      <c r="I23" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>481d4bc, e307a78, ed3573c, e6f8b8c feat(web); dd24095 refactor(web) — feature/driver-ui</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Dashboard with zone and online toggle (locked during a trip); request feed with accept; active trip screen with transition-driven buttons; trip history with cash collection</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs: finalise SRS, architecture and tracker for release
The SRS is baselined as v0.5 with no requirement changed; ARCHITECTURE (1.0) and the ERD (1.0) record that the implementation matches them. ADR-0001…0013 move from Proposed to Accepted now that each decision is built and tested.

In the tracker, a requirement becomes Verified when every linked test case passes: 101 are Verified. TC-34 (forced 500), TC-36 (fresh-clone Docker run), TC-45 (money inspection) and TC-46 (load smoke) now pass; only the UI walkthrough TC-41 remains, so the usability requirements stay Implemented. T-23 and T-26 are done; T-24 (AI Usage section) and T-25 (live URL) are in progress.
</commit_message>
<xml_diff>
--- a/docs/DhakaPool_SRS_Tracker.xlsx
+++ b/docs/DhakaPool_SRS_Tracker.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25 — Phase 9 (feature/driver-ui): driver dashboard, request feed, active trip management, trip history</t>
+          <t>2026-09-25 — Phase 10 (pre-release): fresh-clone fixes, load smoke test, README, scaling notes, deployment configuration; requirements with passing tests marked Verified</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="M2" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N2" s="16" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="M3" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N3" s="16" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="M4" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N4" s="16" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="M5" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N5" s="16" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="M6" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N6" s="16" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N7" s="16" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="M9" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N9" s="16" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="M10" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N10" s="16" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="M11" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N11" s="16" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="M12" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N12" s="16" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="M13" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N13" s="16" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="M14" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N14" s="16" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="M16" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N16" s="16" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="M17" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N17" s="16" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="M18" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N18" s="16" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="M19" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N19" s="16" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="M20" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N20" s="16" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="M21" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N21" s="16" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="M22" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N22" s="16" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="M23" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N23" s="16" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="M24" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N24" s="16" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="M25" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N25" s="16" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="M26" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N26" s="16" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="M27" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N27" s="16" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="M28" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N28" s="16" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M29" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N29" s="16" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="M30" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N30" s="16" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="M31" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N31" s="16" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="M32" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N32" s="16" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="M33" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N33" s="16" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="M34" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N34" s="16" t="inlineStr">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="M35" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N35" s="16" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="M36" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N36" s="16" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="M37" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N37" s="16" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="M38" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N38" s="16" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="M39" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N39" s="16" t="inlineStr">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="M40" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N40" s="16" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="M41" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="M42" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N42" s="16" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="M43" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N43" s="16" t="inlineStr">
@@ -5222,7 +5222,7 @@
       </c>
       <c r="M44" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N44" s="16" t="inlineStr">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="M45" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N45" s="16" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="M46" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N46" s="16" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="M47" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N47" s="16" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="M48" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N48" s="16" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="M49" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N49" s="16" t="inlineStr">
@@ -5688,7 +5688,7 @@
       </c>
       <c r="M50" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N50" s="16" t="inlineStr">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="M51" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N51" s="16" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="M52" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N52" s="16" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M53" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N53" s="16" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="M54" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N54" s="16" t="inlineStr">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="M55" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N55" s="16" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="M56" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N56" s="16" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="M57" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N57" s="16" t="inlineStr">
@@ -6304,7 +6304,7 @@
       </c>
       <c r="M58" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N58" s="16" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="M59" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N59" s="16" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="M60" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N60" s="16" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="M61" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N61" s="16" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="M62" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N62" s="16" t="inlineStr">
@@ -6689,7 +6689,7 @@
       </c>
       <c r="M63" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N63" s="16" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="M64" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N64" s="16" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="M65" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N65" s="16" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="M66" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N66" s="16" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="M67" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N67" s="16" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="M68" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N68" s="16" t="inlineStr">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="M69" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N69" s="16" t="inlineStr">
@@ -7228,7 +7228,7 @@
       </c>
       <c r="M70" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N70" s="16" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="M71" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N71" s="16" t="inlineStr">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="M72" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N72" s="16" t="inlineStr">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="M73" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N73" s="16" t="inlineStr">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="M74" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N74" s="16" t="inlineStr">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="M75" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N75" s="16" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="M76" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N76" s="16" t="inlineStr">
@@ -7767,7 +7767,7 @@
       </c>
       <c r="M77" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N77" s="16" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="M78" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N78" s="16" t="inlineStr">
@@ -7925,7 +7925,7 @@
       </c>
       <c r="M79" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N79" s="16" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="M80" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N80" s="16" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="M81" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N81" s="16" t="inlineStr">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="M82" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N82" s="16" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="M83" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N83" s="16" t="inlineStr">
@@ -8310,7 +8310,7 @@
       </c>
       <c r="M84" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N84" s="16" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="M85" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N85" s="16" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="M86" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N86" s="16" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="M87" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N87" s="16" t="inlineStr">
@@ -8618,7 +8618,7 @@
       </c>
       <c r="M88" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N88" s="16" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="M89" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N89" s="16" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="M90" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N90" s="16" t="inlineStr">
@@ -8849,7 +8849,7 @@
       </c>
       <c r="M91" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N91" s="16" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="M92" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N92" s="16" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="M93" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N93" s="16" t="inlineStr">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="M94" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N94" s="16" t="inlineStr">
@@ -9157,7 +9157,7 @@
       </c>
       <c r="M95" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
@@ -9234,7 +9234,7 @@
       </c>
       <c r="M96" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N96" s="16" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="M97" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
@@ -9388,10 +9388,14 @@
       </c>
       <c r="M98" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N98" s="16" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N98" s="16" t="inlineStr">
+        <is>
+          <t>npm run load:smoke: p95 26.5 ms, 0 failed (TC-46) — pre-release</t>
+        </is>
+      </c>
       <c r="O98" s="16" t="inlineStr"/>
       <c r="P98" s="4">
         <f>","&amp;SUBSTITUTE(F98," ","")&amp;","</f>
@@ -10077,7 +10081,7 @@
       </c>
       <c r="M107" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
@@ -10227,7 +10231,7 @@
       </c>
       <c r="M109" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
@@ -10300,10 +10304,14 @@
       </c>
       <c r="M110" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N110" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N110" s="16" t="inlineStr">
+        <is>
+          <t>render.yaml, apps/web/vercel.json, README Deployment; Docker Compose fallback verified (TC-36) — pre-release</t>
+        </is>
+      </c>
       <c r="O110" s="16" t="inlineStr"/>
       <c r="P110" s="4">
         <f>","&amp;SUBSTITUTE(F110," ","")&amp;","</f>
@@ -10373,7 +10381,7 @@
       </c>
       <c r="M111" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
@@ -10592,7 +10600,7 @@
       </c>
       <c r="M114" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N114" s="16" t="inlineStr">
@@ -10669,7 +10677,7 @@
       </c>
       <c r="M115" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
@@ -10815,12 +10823,12 @@
       </c>
       <c r="M117" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>npm test at root and in Docker (docker compose run --rm api npm test)</t>
+          <t>npm test at the root; docker compose run --rm api npm test (231 passing in a fresh clone) — pre-release</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr"/>
@@ -11107,10 +11115,14 @@
       </c>
       <c r="M121" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N121" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N121" s="16" t="inlineStr">
+        <is>
+          <t>Vercel Hobby, Render free, Supabase free; Railway rejected because its free plan cannot run a service — pre-release</t>
+        </is>
+      </c>
       <c r="O121" s="16" t="inlineStr"/>
       <c r="P121" s="4">
         <f>","&amp;SUBSTITUTE(F121," ","")&amp;","</f>
@@ -11322,10 +11334,14 @@
       </c>
       <c r="M124" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N124" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N124" s="16" t="inlineStr">
+        <is>
+          <t>README 'Tech stack and why' table, one ADR per choice — pre-release</t>
+        </is>
+      </c>
       <c r="O124" s="16" t="inlineStr"/>
       <c r="P124" s="4">
         <f>","&amp;SUBSTITUTE(F124," ","")&amp;","</f>
@@ -11391,10 +11407,14 @@
       </c>
       <c r="M125" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N125" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N125" s="16" t="inlineStr">
+        <is>
+          <t>master and pre-release exist; release/v1.0.0 is cut in the release step — pre-release</t>
+        </is>
+      </c>
       <c r="O125" s="16" t="inlineStr"/>
       <c r="P125" s="4">
         <f>","&amp;SUBSTITUTE(F125," ","")&amp;","</f>
@@ -11460,12 +11480,12 @@
       </c>
       <c r="M126" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N126" s="16" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md §3–4, §12; docs/ERD.md §1</t>
+          <t>feature/* branches merged through PRs #1–#10</t>
         </is>
       </c>
       <c r="O126" s="16" t="inlineStr"/>
@@ -11533,12 +11553,12 @@
       </c>
       <c r="M127" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N127" s="16" t="inlineStr">
         <is>
-          <t>docs/adr/0001–0012 (README summary pending, T-24)</t>
+          <t>Every commit follows &lt;type&gt;(&lt;scope&gt;): &lt;description&gt; (checked with git log; only GitHub's 'Initial commit' differs)</t>
         </is>
       </c>
       <c r="O127" s="16" t="inlineStr"/>
@@ -11606,10 +11626,14 @@
       </c>
       <c r="M128" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N128" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N128" s="16" t="inlineStr">
+        <is>
+          <t>Incremental commits across 13 feature branches, each merged when it worked</t>
+        </is>
+      </c>
       <c r="O128" s="16" t="inlineStr"/>
       <c r="P128" s="4">
         <f>","&amp;SUBSTITUTE(F128," ","")&amp;","</f>
@@ -11679,10 +11703,14 @@
       </c>
       <c r="M129" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N129" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N129" s="16" t="inlineStr">
+        <is>
+          <t>README (8bbd6f6); AI Usage section and video link still to add — pre-release</t>
+        </is>
+      </c>
       <c r="O129" s="16" t="inlineStr"/>
       <c r="P129" s="4">
         <f>","&amp;SUBSTITUTE(F129," ","")&amp;","</f>
@@ -11748,12 +11776,12 @@
       </c>
       <c r="M130" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N130" s="16" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md §3–4, §12; docs/ERD.md §1</t>
+          <t>docs/ARCHITECTURE.md §3–4, docs/ERD.md §1, both embedded in the README</t>
         </is>
       </c>
       <c r="O130" s="16" t="inlineStr"/>
@@ -11821,12 +11849,12 @@
       </c>
       <c r="M131" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N131" s="16" t="inlineStr">
         <is>
-          <t>docs/adr/0001–0012 (README summary pending, T-24)</t>
+          <t>README 'Tech stack and why' + docs/adr/0001–0013 (all Accepted)</t>
         </is>
       </c>
       <c r="O131" s="16" t="inlineStr"/>
@@ -11894,10 +11922,14 @@
       </c>
       <c r="M132" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N132" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N132" s="16" t="inlineStr">
+        <is>
+          <t>Drafted; awaiting the author's wording — pre-release</t>
+        </is>
+      </c>
       <c r="O132" s="16" t="inlineStr"/>
       <c r="P132" s="4">
         <f>","&amp;SUBSTITUTE(F132," ","")&amp;","</f>
@@ -11967,7 +11999,7 @@
       </c>
       <c r="M133" s="15" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N133" s="16" t="inlineStr">
@@ -12040,10 +12072,14 @@
       </c>
       <c r="M134" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N134" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N134" s="16" t="inlineStr">
+        <is>
+          <t>The six PRD §12 areas are tested (README 'Tests'; TC-01…TC-06 passing)</t>
+        </is>
+      </c>
       <c r="O134" s="16" t="inlineStr"/>
       <c r="P134" s="4">
         <f>","&amp;SUBSTITUTE(F134," ","")&amp;","</f>
@@ -12113,10 +12149,14 @@
       </c>
       <c r="M135" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N135" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="N135" s="16" t="inlineStr">
+        <is>
+          <t>Deployment configuration and steps (7ce300f); URL added once live — pre-release</t>
+        </is>
+      </c>
       <c r="O135" s="16" t="inlineStr"/>
       <c r="P135" s="4">
         <f>","&amp;SUBSTITUTE(F135," ","")&amp;","</f>
@@ -12251,10 +12291,14 @@
       </c>
       <c r="M137" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N137" s="16" t="inlineStr"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N137" s="16" t="inlineStr">
+        <is>
+          <t>Free tiers only; .env git-ignored; .env.example has placeholders only</t>
+        </is>
+      </c>
       <c r="O137" s="16" t="inlineStr"/>
       <c r="P137" s="4">
         <f>","&amp;SUBSTITUTE(F137," ","")&amp;","</f>
@@ -12320,12 +12364,12 @@
       </c>
       <c r="M138" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N138" s="16" t="inlineStr">
         <is>
-          <t>SRS v0.2 revision 2026-09-24</t>
+          <t>No queue, cache, microservice or Kubernetes (README, ADR-0001); docs/SCALING.md says when each would be worth it</t>
         </is>
       </c>
       <c r="O138" s="16" t="inlineStr"/>
@@ -12397,12 +12441,12 @@
       </c>
       <c r="M139" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N139" s="16" t="inlineStr">
         <is>
-          <t>Personas in seed and test helpers — feature/db-schema</t>
+          <t>Personas in seed, tests, README and UI (TC-37)</t>
         </is>
       </c>
       <c r="O139" s="16" t="n"/>
@@ -12470,10 +12514,14 @@
       </c>
       <c r="M140" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N140" s="16" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N140" s="16" t="inlineStr">
+        <is>
+          <t>README 'Concurrency: the last-seat problem' — pre-release</t>
+        </is>
+      </c>
       <c r="O140" s="16" t="n"/>
       <c r="P140" s="4">
         <f>","&amp;SUBSTITUTE(F140," ","")&amp;","</f>
@@ -12539,10 +12587,14 @@
       </c>
       <c r="M141" s="15" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="N141" s="16" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="N141" s="16" t="inlineStr">
+        <is>
+          <t>docs/SCALING.md (3228d36) — pre-release</t>
+        </is>
+      </c>
       <c r="O141" s="16" t="n"/>
       <c r="P141" s="4">
         <f>","&amp;SUBSTITUTE(F141," ","")&amp;","</f>
@@ -12608,12 +12660,12 @@
       </c>
       <c r="M142" s="15" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="N142" s="16" t="inlineStr">
         <is>
-          <t>SRS v0.2 revision 2026-09-24</t>
+          <t>SRS v0.5 baseline; tracker updated in every branch</t>
         </is>
       </c>
       <c r="O142" s="16" t="n"/>
@@ -14664,17 +14716,17 @@
       </c>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>Written</t>
+          <t>Passing</t>
         </is>
       </c>
       <c r="J35" s="16" t="inlineStr">
         <is>
-          <t>apps/api/test/app.test.ts (404, malformed JSON, requestId); 409/500 cases added with later modules</t>
+          <t>apps/api/test/app.test.ts (404, malformed JSON, forced 500 without details, requestId); 409/422 across the module tests</t>
         </is>
       </c>
       <c r="K35" s="16" t="inlineStr">
         <is>
-          <t>2026-09-24 passing</t>
+          <t>2026-09-25 passing</t>
         </is>
       </c>
     </row>
@@ -14778,11 +14830,19 @@
       </c>
       <c r="I37" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J37" s="16" t="inlineStr"/>
-      <c r="K37" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J37" s="16" t="inlineStr">
+        <is>
+          <t>Manual: fresh clone of pre-release, cp .env.example .env, docker compose up --build → db, api, web healthy; migrations + seed applied; personas sign in; 231 API tests pass inside Docker</t>
+        </is>
+      </c>
+      <c r="K37" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-25 passing (Docker)</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="33" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
@@ -15275,11 +15335,19 @@
       </c>
       <c r="I46" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J46" s="16" t="inlineStr"/>
-      <c r="K46" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J46" s="16" t="inlineStr">
+        <is>
+          <t>Inspection: every money column is BigInt (schema.prisma; Decimal only for zone lat/lng); fare arithmetic is integer (domain/money.ts roundHalfUpDiv); display only via formatPaisa</t>
+        </is>
+      </c>
+      <c r="K46" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-25 passing (inspection)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="33" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
@@ -15324,11 +15392,19 @@
       </c>
       <c r="I47" s="15" t="inlineStr">
         <is>
-          <t>Not Written</t>
-        </is>
-      </c>
-      <c r="J47" s="16" t="inlineStr"/>
-      <c r="K47" s="16" t="inlineStr"/>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="inlineStr">
+        <is>
+          <t>scripts/load-smoke.mjs (npm run load:smoke): 20 users × 60 s, 87,367 requests, 0 failed, p95 26.5 ms</t>
+        </is>
+      </c>
+      <c r="K47" s="16" t="inlineStr">
+        <is>
+          <t>2026-09-25 passing (fresh Docker stack)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
@@ -19035,11 +19111,19 @@
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H24" s="16" t="inlineStr"/>
-      <c r="I24" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>67fb6fb fix(env), d1d7715 fix(docker), 5d65a4c fix(api), fc2f4f1 fix(db); d5293e7 test(perf); ca81bb9 test(api) — pre-release</t>
+        </is>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Fresh-clone Docker run (TC-36) found the unquoted demo password and the missing OpenSSL; deployment review found the proxy hop count and the unused DIRECT_URL. Load smoke p95 26.5 ms. Browser walkthrough (TC-41) still to do.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -19072,11 +19156,19 @@
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H25" s="16" t="inlineStr"/>
-      <c r="I25" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>8bbd6f6 docs(readme) — pre-release</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Everything except the AI Usage section (awaiting the author's wording) and the demo video link (release)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
@@ -19109,11 +19201,19 @@
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H26" s="16" t="inlineStr"/>
-      <c r="I26" s="16" t="inlineStr"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>7ce300f build(deploy) — pre-release</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>render.yaml + apps/web/vercel.json + README steps; Railway's free plan cannot run a service, so Render (ADR-0009 fallback). Live URL once the accounts are set up</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
@@ -19146,11 +19246,19 @@
       </c>
       <c r="G27" s="15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H27" s="16" t="inlineStr"/>
-      <c r="I27" s="16" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>3228d36 docs(scaling) — pre-release</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>docs/SCALING.md with load estimate, target architecture and diagram</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="33" customHeight="1">
       <c r="A28" s="14" t="inlineStr">

</xml_diff>